<commit_message>
NS 3451 level: minLevel on code-lookup, Nivå 2 / Nivå 3+ on the Krav editor
A listed NS 3451 code shorter than minLevel (2 or 3 digits) fails with
finding code `level`; unset keeps today's behaviour. Carried through
resolveLookup (so the Kilde value table, the walk candidates and the
standard option judge against it), lint (min-level-invalid, a warning on
another list), the JSON schema, the xlsx Klassifikasjon sheet (column Nivå),
the report's requirement column and the Krav data line, whose examples follow
the level. IDS export and the POFIN default are unchanged.

Selftest 535 (13 new).

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/examples/eks-config-template.xlsx
+++ b/examples/eks-config-template.xlsx
@@ -2337,32 +2337,22 @@
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t xml:space="preserve">Kildetype</t>
+          <t xml:space="preserve">Nivå</t>
         </is>
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t xml:space="preserve">rules[].check.source</t>
+          <t xml:space="preserve">rules[].check.minLevel</t>
         </is>
       </c>
       <c r="D107" t="inlineStr">
         <is>
-          <t xml:space="preserve">source kind</t>
-        </is>
-      </c>
-      <c r="E107" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
-        </is>
-      </c>
-      <c r="F107" t="inlineStr">
-        <is>
-          <t xml:space="preserve">attribute, property, classification, material, progressCode</t>
+          <t xml:space="preserve">number</t>
         </is>
       </c>
       <c r="G107" t="inlineStr">
         <is>
-          <t xml:space="preserve">attribute</t>
+          <t xml:space="preserve">3</t>
         </is>
       </c>
     </row>
@@ -2374,22 +2364,32 @@
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t xml:space="preserve">Attributt</t>
+          <t xml:space="preserve">Kildetype</t>
         </is>
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t xml:space="preserve">rules[].check.source.attribute</t>
+          <t xml:space="preserve">rules[].check.source</t>
         </is>
       </c>
       <c r="D108" t="inlineStr">
         <is>
-          <t xml:space="preserve">text</t>
+          <t xml:space="preserve">source kind</t>
+        </is>
+      </c>
+      <c r="E108" t="inlineStr">
+        <is>
+          <t xml:space="preserve">yes</t>
+        </is>
+      </c>
+      <c r="F108" t="inlineStr">
+        <is>
+          <t xml:space="preserve">attribute, property, classification, material, progressCode</t>
         </is>
       </c>
       <c r="G108" t="inlineStr">
         <is>
-          <t xml:space="preserve">Name</t>
+          <t xml:space="preserve">attribute</t>
         </is>
       </c>
     </row>
@@ -2401,12 +2401,12 @@
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t xml:space="preserve">Egenskapssett</t>
+          <t xml:space="preserve">Attributt</t>
         </is>
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t xml:space="preserve">rules[].check.source.property.propertySet</t>
+          <t xml:space="preserve">rules[].check.source.attribute</t>
         </is>
       </c>
       <c r="D109" t="inlineStr">
@@ -2416,7 +2416,7 @@
       </c>
       <c r="G109" t="inlineStr">
         <is>
-          <t xml:space="preserve">EKS_Project</t>
+          <t xml:space="preserve">Name</t>
         </is>
       </c>
     </row>
@@ -2428,12 +2428,12 @@
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t xml:space="preserve">Egenskapsnavn</t>
+          <t xml:space="preserve">Egenskapssett</t>
         </is>
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t xml:space="preserve">rules[].check.source.property.name</t>
+          <t xml:space="preserve">rules[].check.source.property.propertySet</t>
         </is>
       </c>
       <c r="D110" t="inlineStr">
@@ -2443,7 +2443,7 @@
       </c>
       <c r="G110" t="inlineStr">
         <is>
-          <t xml:space="preserve">MMI</t>
+          <t xml:space="preserve">EKS_Project</t>
         </is>
       </c>
     </row>
@@ -2455,12 +2455,12 @@
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t xml:space="preserve">System</t>
+          <t xml:space="preserve">Egenskapsnavn</t>
         </is>
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t xml:space="preserve">rules[].check.source.classification.system</t>
+          <t xml:space="preserve">rules[].check.source.property.name</t>
         </is>
       </c>
       <c r="D111" t="inlineStr">
@@ -2470,7 +2470,7 @@
       </c>
       <c r="G111" t="inlineStr">
         <is>
-          <t xml:space="preserve">NS 3451</t>
+          <t xml:space="preserve">MMI</t>
         </is>
       </c>
     </row>
@@ -2482,12 +2482,12 @@
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t xml:space="preserve">Uttrekk (regex)</t>
+          <t xml:space="preserve">System</t>
         </is>
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t xml:space="preserve">rules[].check.extract</t>
+          <t xml:space="preserve">rules[].check.source.classification.system</t>
         </is>
       </c>
       <c r="D112" t="inlineStr">
@@ -2495,14 +2495,9 @@
           <t xml:space="preserve">text</t>
         </is>
       </c>
-      <c r="E112" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
-        </is>
-      </c>
       <c r="G112" t="inlineStr">
         <is>
-          <t xml:space="preserve">^([A-Z]{2,3})-\d{2}$</t>
+          <t xml:space="preserve">NS 3451</t>
         </is>
       </c>
     </row>
@@ -2514,17 +2509,17 @@
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t xml:space="preserve">Aktiv</t>
+          <t xml:space="preserve">Uttrekk (regex)</t>
         </is>
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t xml:space="preserve">rules[].enabled</t>
+          <t xml:space="preserve">rules[].check.extract</t>
         </is>
       </c>
       <c r="D113" t="inlineStr">
         <is>
-          <t xml:space="preserve">TRUE / FALSE</t>
+          <t xml:space="preserve">text</t>
         </is>
       </c>
       <c r="E113" t="inlineStr">
@@ -2532,14 +2527,9 @@
           <t xml:space="preserve">yes</t>
         </is>
       </c>
-      <c r="F113" t="inlineStr">
-        <is>
-          <t xml:space="preserve">TRUE, FALSE</t>
-        </is>
-      </c>
       <c r="G113" t="inlineStr">
         <is>
-          <t xml:space="preserve">TRUE</t>
+          <t xml:space="preserve">^([A-Z]{2,3})-\d{2}$</t>
         </is>
       </c>
     </row>
@@ -2551,22 +2541,32 @@
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t xml:space="preserve">Utvalg</t>
+          <t xml:space="preserve">Aktiv</t>
         </is>
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t xml:space="preserve">rules[].select</t>
+          <t xml:space="preserve">rules[].enabled</t>
         </is>
       </c>
       <c r="D114" t="inlineStr">
         <is>
-          <t xml:space="preserve">JSON</t>
+          <t xml:space="preserve">TRUE / FALSE</t>
+        </is>
+      </c>
+      <c r="E114" t="inlineStr">
+        <is>
+          <t xml:space="preserve">yes</t>
+        </is>
+      </c>
+      <c r="F114" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TRUE, FALSE</t>
         </is>
       </c>
       <c r="G114" t="inlineStr">
         <is>
-          <t xml:space="preserve">{"entity":{"group":"physicalElement"}}</t>
+          <t xml:space="preserve">TRUE</t>
         </is>
       </c>
     </row>
@@ -2578,49 +2578,44 @@
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t xml:space="preserve">Instruksjon</t>
+          <t xml:space="preserve">Utvalg</t>
         </is>
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t xml:space="preserve">rules[].instructions</t>
+          <t xml:space="preserve">rules[].select</t>
         </is>
       </c>
       <c r="D115" t="inlineStr">
         <is>
-          <t xml:space="preserve">text</t>
+          <t xml:space="preserve">JSON</t>
+        </is>
+      </c>
+      <c r="G115" t="inlineStr">
+        <is>
+          <t xml:space="preserve">{"entity":{"group":"physicalElement"}}</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t xml:space="preserve">MMI</t>
+          <t xml:space="preserve">Klassifikasjon</t>
         </is>
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t xml:space="preserve">ID</t>
+          <t xml:space="preserve">Instruksjon</t>
         </is>
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t xml:space="preserve">rules[].id</t>
+          <t xml:space="preserve">rules[].instructions</t>
         </is>
       </c>
       <c r="D116" t="inlineStr">
         <is>
           <t xml:space="preserve">text</t>
-        </is>
-      </c>
-      <c r="E116" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
-        </is>
-      </c>
-      <c r="G116" t="inlineStr">
-        <is>
-          <t xml:space="preserve">progress-code</t>
         </is>
       </c>
     </row>
@@ -2632,12 +2627,12 @@
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t xml:space="preserve">Navn</t>
+          <t xml:space="preserve">ID</t>
         </is>
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t xml:space="preserve">rules[].name</t>
+          <t xml:space="preserve">rules[].id</t>
         </is>
       </c>
       <c r="D117" t="inlineStr">
@@ -2652,7 +2647,7 @@
       </c>
       <c r="G117" t="inlineStr">
         <is>
-          <t xml:space="preserve">MMI</t>
+          <t xml:space="preserve">progress-code</t>
         </is>
       </c>
     </row>
@@ -2664,17 +2659,27 @@
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t xml:space="preserve">Beskrivelse</t>
+          <t xml:space="preserve">Navn</t>
         </is>
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t xml:space="preserve">rules[].description</t>
+          <t xml:space="preserve">rules[].name</t>
         </is>
       </c>
       <c r="D118" t="inlineStr">
         <is>
           <t xml:space="preserve">text</t>
+        </is>
+      </c>
+      <c r="E118" t="inlineStr">
+        <is>
+          <t xml:space="preserve">yes</t>
+        </is>
+      </c>
+      <c r="G118" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MMI</t>
         </is>
       </c>
     </row>
@@ -2686,22 +2691,17 @@
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t xml:space="preserve">Referanse</t>
+          <t xml:space="preserve">Beskrivelse</t>
         </is>
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t xml:space="preserve">rules[].reference</t>
+          <t xml:space="preserve">rules[].description</t>
         </is>
       </c>
       <c r="D119" t="inlineStr">
         <is>
           <t xml:space="preserve">text</t>
-        </is>
-      </c>
-      <c r="G119" t="inlineStr">
-        <is>
-          <t xml:space="preserve">BEP §6.12</t>
         </is>
       </c>
     </row>
@@ -2713,32 +2713,22 @@
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t xml:space="preserve">Kildetype</t>
+          <t xml:space="preserve">Referanse</t>
         </is>
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t xml:space="preserve">rules[].check.source</t>
+          <t xml:space="preserve">rules[].reference</t>
         </is>
       </c>
       <c r="D120" t="inlineStr">
         <is>
-          <t xml:space="preserve">source kind</t>
-        </is>
-      </c>
-      <c r="E120" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
-        </is>
-      </c>
-      <c r="F120" t="inlineStr">
-        <is>
-          <t xml:space="preserve">attribute, property, classification, material, progressCode</t>
+          <t xml:space="preserve">text</t>
         </is>
       </c>
       <c r="G120" t="inlineStr">
         <is>
-          <t xml:space="preserve">property</t>
+          <t xml:space="preserve">BEP §6.12</t>
         </is>
       </c>
     </row>
@@ -2750,22 +2740,32 @@
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t xml:space="preserve">Attributt</t>
+          <t xml:space="preserve">Kildetype</t>
         </is>
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t xml:space="preserve">rules[].check.source.attribute</t>
+          <t xml:space="preserve">rules[].check.source</t>
         </is>
       </c>
       <c r="D121" t="inlineStr">
         <is>
-          <t xml:space="preserve">text</t>
+          <t xml:space="preserve">source kind</t>
+        </is>
+      </c>
+      <c r="E121" t="inlineStr">
+        <is>
+          <t xml:space="preserve">yes</t>
+        </is>
+      </c>
+      <c r="F121" t="inlineStr">
+        <is>
+          <t xml:space="preserve">attribute, property, classification, material, progressCode</t>
         </is>
       </c>
       <c r="G121" t="inlineStr">
         <is>
-          <t xml:space="preserve">Name</t>
+          <t xml:space="preserve">property</t>
         </is>
       </c>
     </row>
@@ -2777,12 +2777,12 @@
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t xml:space="preserve">Egenskapssett</t>
+          <t xml:space="preserve">Attributt</t>
         </is>
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t xml:space="preserve">rules[].check.source.property.propertySet</t>
+          <t xml:space="preserve">rules[].check.source.attribute</t>
         </is>
       </c>
       <c r="D122" t="inlineStr">
@@ -2792,7 +2792,7 @@
       </c>
       <c r="G122" t="inlineStr">
         <is>
-          <t xml:space="preserve">EKS_Project</t>
+          <t xml:space="preserve">Name</t>
         </is>
       </c>
     </row>
@@ -2804,12 +2804,12 @@
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t xml:space="preserve">Egenskapsnavn</t>
+          <t xml:space="preserve">Egenskapssett</t>
         </is>
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t xml:space="preserve">rules[].check.source.property.name</t>
+          <t xml:space="preserve">rules[].check.source.property.propertySet</t>
         </is>
       </c>
       <c r="D123" t="inlineStr">
@@ -2819,7 +2819,7 @@
       </c>
       <c r="G123" t="inlineStr">
         <is>
-          <t xml:space="preserve">MMI</t>
+          <t xml:space="preserve">EKS_Project</t>
         </is>
       </c>
     </row>
@@ -2831,12 +2831,12 @@
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t xml:space="preserve">System</t>
+          <t xml:space="preserve">Egenskapsnavn</t>
         </is>
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t xml:space="preserve">rules[].check.source.classification.system</t>
+          <t xml:space="preserve">rules[].check.source.property.name</t>
         </is>
       </c>
       <c r="D124" t="inlineStr">
@@ -2846,7 +2846,7 @@
       </c>
       <c r="G124" t="inlineStr">
         <is>
-          <t xml:space="preserve">NS 3451</t>
+          <t xml:space="preserve">MMI</t>
         </is>
       </c>
     </row>
@@ -2858,12 +2858,12 @@
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t xml:space="preserve">Uttrekk (regex)</t>
+          <t xml:space="preserve">System</t>
         </is>
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t xml:space="preserve">rules[].check.extract</t>
+          <t xml:space="preserve">rules[].check.source.classification.system</t>
         </is>
       </c>
       <c r="D125" t="inlineStr">
@@ -2871,14 +2871,9 @@
           <t xml:space="preserve">text</t>
         </is>
       </c>
-      <c r="E125" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
-        </is>
-      </c>
       <c r="G125" t="inlineStr">
         <is>
-          <t xml:space="preserve">^(\d{3})$</t>
+          <t xml:space="preserve">NS 3451</t>
         </is>
       </c>
     </row>
@@ -2890,17 +2885,17 @@
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t xml:space="preserve">Aktiv</t>
+          <t xml:space="preserve">Uttrekk (regex)</t>
         </is>
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t xml:space="preserve">rules[].enabled</t>
+          <t xml:space="preserve">rules[].check.extract</t>
         </is>
       </c>
       <c r="D126" t="inlineStr">
         <is>
-          <t xml:space="preserve">TRUE / FALSE</t>
+          <t xml:space="preserve">text</t>
         </is>
       </c>
       <c r="E126" t="inlineStr">
@@ -2908,14 +2903,9 @@
           <t xml:space="preserve">yes</t>
         </is>
       </c>
-      <c r="F126" t="inlineStr">
-        <is>
-          <t xml:space="preserve">TRUE, FALSE</t>
-        </is>
-      </c>
       <c r="G126" t="inlineStr">
         <is>
-          <t xml:space="preserve">TRUE</t>
+          <t xml:space="preserve">^(\d{3})$</t>
         </is>
       </c>
     </row>
@@ -2927,22 +2917,32 @@
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t xml:space="preserve">Utvalg</t>
+          <t xml:space="preserve">Aktiv</t>
         </is>
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t xml:space="preserve">rules[].select</t>
+          <t xml:space="preserve">rules[].enabled</t>
         </is>
       </c>
       <c r="D127" t="inlineStr">
         <is>
-          <t xml:space="preserve">JSON</t>
+          <t xml:space="preserve">TRUE / FALSE</t>
+        </is>
+      </c>
+      <c r="E127" t="inlineStr">
+        <is>
+          <t xml:space="preserve">yes</t>
+        </is>
+      </c>
+      <c r="F127" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TRUE, FALSE</t>
         </is>
       </c>
       <c r="G127" t="inlineStr">
         <is>
-          <t xml:space="preserve">{"entity":{"group":"physicalElement"}}</t>
+          <t xml:space="preserve">TRUE</t>
         </is>
       </c>
     </row>
@@ -2954,49 +2954,44 @@
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t xml:space="preserve">Instruksjon</t>
+          <t xml:space="preserve">Utvalg</t>
         </is>
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t xml:space="preserve">rules[].instructions</t>
+          <t xml:space="preserve">rules[].select</t>
         </is>
       </c>
       <c r="D128" t="inlineStr">
         <is>
-          <t xml:space="preserve">text</t>
+          <t xml:space="preserve">JSON</t>
+        </is>
+      </c>
+      <c r="G128" t="inlineStr">
+        <is>
+          <t xml:space="preserve">{"entity":{"group":"physicalElement"}}</t>
         </is>
       </c>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t xml:space="preserve">MMI-koder</t>
+          <t xml:space="preserve">MMI</t>
         </is>
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t xml:space="preserve">Kode</t>
+          <t xml:space="preserve">Instruksjon</t>
         </is>
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t xml:space="preserve">rules[].check.codes[].code</t>
+          <t xml:space="preserve">rules[].instructions</t>
         </is>
       </c>
       <c r="D129" t="inlineStr">
         <is>
           <t xml:space="preserve">text</t>
-        </is>
-      </c>
-      <c r="E129" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
-        </is>
-      </c>
-      <c r="G129" t="inlineStr">
-        <is>
-          <t xml:space="preserve">300</t>
         </is>
       </c>
     </row>
@@ -3008,12 +3003,12 @@
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t xml:space="preserve">Navn</t>
+          <t xml:space="preserve">Kode</t>
         </is>
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t xml:space="preserve">rules[].check.codes[].name</t>
+          <t xml:space="preserve">rules[].check.codes[].code</t>
         </is>
       </c>
       <c r="D130" t="inlineStr">
@@ -3028,7 +3023,7 @@
       </c>
       <c r="G130" t="inlineStr">
         <is>
-          <t xml:space="preserve">Detaljprosjektert</t>
+          <t xml:space="preserve">300</t>
         </is>
       </c>
     </row>
@@ -3040,12 +3035,12 @@
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t xml:space="preserve">Fase</t>
+          <t xml:space="preserve">Navn</t>
         </is>
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t xml:space="preserve">rules[].check.codes[].phase</t>
+          <t xml:space="preserve">rules[].check.codes[].name</t>
         </is>
       </c>
       <c r="D131" t="inlineStr">
@@ -3053,26 +3048,31 @@
           <t xml:space="preserve">text</t>
         </is>
       </c>
+      <c r="E131" t="inlineStr">
+        <is>
+          <t xml:space="preserve">yes</t>
+        </is>
+      </c>
       <c r="G131" t="inlineStr">
         <is>
-          <t xml:space="preserve">NY</t>
+          <t xml:space="preserve">Detaljprosjektert</t>
         </is>
       </c>
     </row>
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t xml:space="preserve">Kopiobjekt</t>
+          <t xml:space="preserve">MMI-koder</t>
         </is>
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t xml:space="preserve">ID</t>
+          <t xml:space="preserve">Fase</t>
         </is>
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t xml:space="preserve">rules[].id</t>
+          <t xml:space="preserve">rules[].check.codes[].phase</t>
         </is>
       </c>
       <c r="D132" t="inlineStr">
@@ -3080,14 +3080,9 @@
           <t xml:space="preserve">text</t>
         </is>
       </c>
-      <c r="E132" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
-        </is>
-      </c>
       <c r="G132" t="inlineStr">
         <is>
-          <t xml:space="preserve">copy-object</t>
+          <t xml:space="preserve">NY</t>
         </is>
       </c>
     </row>
@@ -3099,12 +3094,12 @@
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t xml:space="preserve">Navn</t>
+          <t xml:space="preserve">ID</t>
         </is>
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t xml:space="preserve">rules[].name</t>
+          <t xml:space="preserve">rules[].id</t>
         </is>
       </c>
       <c r="D133" t="inlineStr">
@@ -3119,7 +3114,7 @@
       </c>
       <c r="G133" t="inlineStr">
         <is>
-          <t xml:space="preserve">Kopiobjekt</t>
+          <t xml:space="preserve">copy-object</t>
         </is>
       </c>
     </row>
@@ -3131,17 +3126,27 @@
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t xml:space="preserve">Beskrivelse</t>
+          <t xml:space="preserve">Navn</t>
         </is>
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t xml:space="preserve">rules[].description</t>
+          <t xml:space="preserve">rules[].name</t>
         </is>
       </c>
       <c r="D134" t="inlineStr">
         <is>
           <t xml:space="preserve">text</t>
+        </is>
+      </c>
+      <c r="E134" t="inlineStr">
+        <is>
+          <t xml:space="preserve">yes</t>
+        </is>
+      </c>
+      <c r="G134" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Kopiobjekt</t>
         </is>
       </c>
     </row>
@@ -3153,22 +3158,17 @@
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t xml:space="preserve">Referanse</t>
+          <t xml:space="preserve">Beskrivelse</t>
         </is>
       </c>
       <c r="C135" t="inlineStr">
         <is>
-          <t xml:space="preserve">rules[].reference</t>
+          <t xml:space="preserve">rules[].description</t>
         </is>
       </c>
       <c r="D135" t="inlineStr">
         <is>
           <t xml:space="preserve">text</t>
-        </is>
-      </c>
-      <c r="G135" t="inlineStr">
-        <is>
-          <t xml:space="preserve">BEP §6.12</t>
         </is>
       </c>
     </row>
@@ -3180,32 +3180,22 @@
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t xml:space="preserve">Kildetype</t>
+          <t xml:space="preserve">Referanse</t>
         </is>
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t xml:space="preserve">rules[].check.source</t>
+          <t xml:space="preserve">rules[].reference</t>
         </is>
       </c>
       <c r="D136" t="inlineStr">
         <is>
-          <t xml:space="preserve">source kind</t>
-        </is>
-      </c>
-      <c r="E136" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
-        </is>
-      </c>
-      <c r="F136" t="inlineStr">
-        <is>
-          <t xml:space="preserve">attribute, property, classification, material, progressCode</t>
+          <t xml:space="preserve">text</t>
         </is>
       </c>
       <c r="G136" t="inlineStr">
         <is>
-          <t xml:space="preserve">property</t>
+          <t xml:space="preserve">BEP §6.12</t>
         </is>
       </c>
     </row>
@@ -3217,22 +3207,32 @@
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t xml:space="preserve">Attributt</t>
+          <t xml:space="preserve">Kildetype</t>
         </is>
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t xml:space="preserve">rules[].check.source.attribute</t>
+          <t xml:space="preserve">rules[].check.source</t>
         </is>
       </c>
       <c r="D137" t="inlineStr">
         <is>
-          <t xml:space="preserve">text</t>
+          <t xml:space="preserve">source kind</t>
+        </is>
+      </c>
+      <c r="E137" t="inlineStr">
+        <is>
+          <t xml:space="preserve">yes</t>
+        </is>
+      </c>
+      <c r="F137" t="inlineStr">
+        <is>
+          <t xml:space="preserve">attribute, property, classification, material, progressCode</t>
         </is>
       </c>
       <c r="G137" t="inlineStr">
         <is>
-          <t xml:space="preserve">Name</t>
+          <t xml:space="preserve">property</t>
         </is>
       </c>
     </row>
@@ -3244,12 +3244,12 @@
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t xml:space="preserve">Egenskapssett</t>
+          <t xml:space="preserve">Attributt</t>
         </is>
       </c>
       <c r="C138" t="inlineStr">
         <is>
-          <t xml:space="preserve">rules[].check.source.property.propertySet</t>
+          <t xml:space="preserve">rules[].check.source.attribute</t>
         </is>
       </c>
       <c r="D138" t="inlineStr">
@@ -3259,7 +3259,7 @@
       </c>
       <c r="G138" t="inlineStr">
         <is>
-          <t xml:space="preserve">EKS_Project</t>
+          <t xml:space="preserve">Name</t>
         </is>
       </c>
     </row>
@@ -3271,12 +3271,12 @@
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t xml:space="preserve">Egenskapsnavn</t>
+          <t xml:space="preserve">Egenskapssett</t>
         </is>
       </c>
       <c r="C139" t="inlineStr">
         <is>
-          <t xml:space="preserve">rules[].check.source.property.name</t>
+          <t xml:space="preserve">rules[].check.source.property.propertySet</t>
         </is>
       </c>
       <c r="D139" t="inlineStr">
@@ -3286,7 +3286,7 @@
       </c>
       <c r="G139" t="inlineStr">
         <is>
-          <t xml:space="preserve">MMI</t>
+          <t xml:space="preserve">EKS_Project</t>
         </is>
       </c>
     </row>
@@ -3298,12 +3298,12 @@
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t xml:space="preserve">System</t>
+          <t xml:space="preserve">Egenskapsnavn</t>
         </is>
       </c>
       <c r="C140" t="inlineStr">
         <is>
-          <t xml:space="preserve">rules[].check.source.classification.system</t>
+          <t xml:space="preserve">rules[].check.source.property.name</t>
         </is>
       </c>
       <c r="D140" t="inlineStr">
@@ -3313,7 +3313,7 @@
       </c>
       <c r="G140" t="inlineStr">
         <is>
-          <t xml:space="preserve">NS 3451</t>
+          <t xml:space="preserve">MMI</t>
         </is>
       </c>
     </row>
@@ -3325,22 +3325,22 @@
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t xml:space="preserve">Kopiverdier</t>
+          <t xml:space="preserve">System</t>
         </is>
       </c>
       <c r="C141" t="inlineStr">
         <is>
-          <t xml:space="preserve">rules[].check.copy</t>
+          <t xml:space="preserve">rules[].check.source.classification.system</t>
         </is>
       </c>
       <c r="D141" t="inlineStr">
         <is>
-          <t xml:space="preserve">list, blank = none</t>
+          <t xml:space="preserve">text</t>
         </is>
       </c>
       <c r="G141" t="inlineStr">
         <is>
-          <t xml:space="preserve">true, ja, kopi</t>
+          <t xml:space="preserve">NS 3451</t>
         </is>
       </c>
     </row>
@@ -3352,12 +3352,12 @@
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t xml:space="preserve">Egne verdier</t>
+          <t xml:space="preserve">Kopiverdier</t>
         </is>
       </c>
       <c r="C142" t="inlineStr">
         <is>
-          <t xml:space="preserve">rules[].check.own</t>
+          <t xml:space="preserve">rules[].check.copy</t>
         </is>
       </c>
       <c r="D142" t="inlineStr">
@@ -3367,7 +3367,7 @@
       </c>
       <c r="G142" t="inlineStr">
         <is>
-          <t xml:space="preserve">false, nei</t>
+          <t xml:space="preserve">true, ja, kopi</t>
         </is>
       </c>
     </row>
@@ -3379,32 +3379,22 @@
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t xml:space="preserve">Aktiv</t>
+          <t xml:space="preserve">Egne verdier</t>
         </is>
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t xml:space="preserve">rules[].enabled</t>
+          <t xml:space="preserve">rules[].check.own</t>
         </is>
       </c>
       <c r="D143" t="inlineStr">
         <is>
-          <t xml:space="preserve">TRUE / FALSE</t>
-        </is>
-      </c>
-      <c r="E143" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
-        </is>
-      </c>
-      <c r="F143" t="inlineStr">
-        <is>
-          <t xml:space="preserve">TRUE, FALSE</t>
+          <t xml:space="preserve">list, blank = none</t>
         </is>
       </c>
       <c r="G143" t="inlineStr">
         <is>
-          <t xml:space="preserve">TRUE</t>
+          <t xml:space="preserve">false, nei</t>
         </is>
       </c>
     </row>
@@ -3416,22 +3406,32 @@
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t xml:space="preserve">Utvalg</t>
+          <t xml:space="preserve">Aktiv</t>
         </is>
       </c>
       <c r="C144" t="inlineStr">
         <is>
-          <t xml:space="preserve">rules[].select</t>
+          <t xml:space="preserve">rules[].enabled</t>
         </is>
       </c>
       <c r="D144" t="inlineStr">
         <is>
-          <t xml:space="preserve">JSON</t>
+          <t xml:space="preserve">TRUE / FALSE</t>
+        </is>
+      </c>
+      <c r="E144" t="inlineStr">
+        <is>
+          <t xml:space="preserve">yes</t>
+        </is>
+      </c>
+      <c r="F144" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TRUE, FALSE</t>
         </is>
       </c>
       <c r="G144" t="inlineStr">
         <is>
-          <t xml:space="preserve">{"entity":{"group":"physicalElement"}}</t>
+          <t xml:space="preserve">TRUE</t>
         </is>
       </c>
     </row>
@@ -3443,44 +3443,44 @@
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t xml:space="preserve">Instruksjon</t>
+          <t xml:space="preserve">Utvalg</t>
         </is>
       </c>
       <c r="C145" t="inlineStr">
         <is>
-          <t xml:space="preserve">rules[].instructions</t>
+          <t xml:space="preserve">rules[].select</t>
         </is>
       </c>
       <c r="D145" t="inlineStr">
         <is>
-          <t xml:space="preserve">text</t>
+          <t xml:space="preserve">JSON</t>
+        </is>
+      </c>
+      <c r="G145" t="inlineStr">
+        <is>
+          <t xml:space="preserve">{"entity":{"group":"physicalElement"}}</t>
         </is>
       </c>
     </row>
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t xml:space="preserve">Etasjeoppsett</t>
+          <t xml:space="preserve">Kopiobjekt</t>
         </is>
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t xml:space="preserve">Fagkode</t>
+          <t xml:space="preserve">Instruksjon</t>
         </is>
       </c>
       <c r="C146" t="inlineStr">
         <is>
-          <t xml:space="preserve">discipline</t>
+          <t xml:space="preserve">rules[].instructions</t>
         </is>
       </c>
       <c r="D146" t="inlineStr">
         <is>
           <t xml:space="preserve">text</t>
-        </is>
-      </c>
-      <c r="G146" t="inlineStr">
-        <is>
-          <t xml:space="preserve">RIB</t>
         </is>
       </c>
     </row>
@@ -3492,12 +3492,12 @@
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t xml:space="preserve">Referanseplan</t>
+          <t xml:space="preserve">Fagkode</t>
         </is>
       </c>
       <c r="C147" t="inlineStr">
         <is>
-          <t xml:space="preserve">plane</t>
+          <t xml:space="preserve">discipline</t>
         </is>
       </c>
       <c r="D147" t="inlineStr">
@@ -3505,19 +3505,9 @@
           <t xml:space="preserve">text</t>
         </is>
       </c>
-      <c r="E147" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
-        </is>
-      </c>
-      <c r="F147" t="inlineStr">
-        <is>
-          <t xml:space="preserve">OKFG, OKBD</t>
-        </is>
-      </c>
       <c r="G147" t="inlineStr">
         <is>
-          <t xml:space="preserve">OKFG</t>
+          <t xml:space="preserve">RIB</t>
         </is>
       </c>
     </row>
@@ -3529,22 +3519,32 @@
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t xml:space="preserve">Toleranse over (mm)</t>
+          <t xml:space="preserve">Referanseplan</t>
         </is>
       </c>
       <c r="C148" t="inlineStr">
         <is>
-          <t xml:space="preserve">tolerance.aboveMm</t>
+          <t xml:space="preserve">plane</t>
         </is>
       </c>
       <c r="D148" t="inlineStr">
         <is>
-          <t xml:space="preserve">mm, blank = no limit</t>
+          <t xml:space="preserve">text</t>
+        </is>
+      </c>
+      <c r="E148" t="inlineStr">
+        <is>
+          <t xml:space="preserve">yes</t>
+        </is>
+      </c>
+      <c r="F148" t="inlineStr">
+        <is>
+          <t xml:space="preserve">OKFG, OKBD</t>
         </is>
       </c>
       <c r="G148" t="inlineStr">
         <is>
-          <t xml:space="preserve">5</t>
+          <t xml:space="preserve">OKFG</t>
         </is>
       </c>
     </row>
@@ -3556,12 +3556,12 @@
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t xml:space="preserve">Toleranse under (mm)</t>
+          <t xml:space="preserve">Toleranse over (mm)</t>
         </is>
       </c>
       <c r="C149" t="inlineStr">
         <is>
-          <t xml:space="preserve">tolerance.belowMm</t>
+          <t xml:space="preserve">tolerance.aboveMm</t>
         </is>
       </c>
       <c r="D149" t="inlineStr">
@@ -3583,12 +3583,12 @@
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t xml:space="preserve">Navnevindu (mm)</t>
+          <t xml:space="preserve">Toleranse under (mm)</t>
         </is>
       </c>
       <c r="C150" t="inlineStr">
         <is>
-          <t xml:space="preserve">nameWindowMm</t>
+          <t xml:space="preserve">tolerance.belowMm</t>
         </is>
       </c>
       <c r="D150" t="inlineStr">
@@ -3598,7 +3598,7 @@
       </c>
       <c r="G150" t="inlineStr">
         <is>
-          <t xml:space="preserve">1000</t>
+          <t xml:space="preserve">5</t>
         </is>
       </c>
     </row>
@@ -3610,22 +3610,22 @@
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t xml:space="preserve">Nærvindu (mm)</t>
+          <t xml:space="preserve">Navnevindu (mm)</t>
         </is>
       </c>
       <c r="C151" t="inlineStr">
         <is>
-          <t xml:space="preserve">nearMm</t>
+          <t xml:space="preserve">nameWindowMm</t>
         </is>
       </c>
       <c r="D151" t="inlineStr">
         <is>
-          <t xml:space="preserve">number</t>
+          <t xml:space="preserve">mm, blank = no limit</t>
         </is>
       </c>
       <c r="G151" t="inlineStr">
         <is>
-          <t xml:space="preserve">200</t>
+          <t xml:space="preserve">1000</t>
         </is>
       </c>
     </row>
@@ -3637,27 +3637,22 @@
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t xml:space="preserve">Alle navn må stemme</t>
+          <t xml:space="preserve">Nærvindu (mm)</t>
         </is>
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t xml:space="preserve">requireAllNames</t>
+          <t xml:space="preserve">nearMm</t>
         </is>
       </c>
       <c r="D152" t="inlineStr">
         <is>
-          <t xml:space="preserve">TRUE / FALSE</t>
-        </is>
-      </c>
-      <c r="F152" t="inlineStr">
-        <is>
-          <t xml:space="preserve">TRUE, FALSE</t>
+          <t xml:space="preserve">number</t>
         </is>
       </c>
       <c r="G152" t="inlineStr">
         <is>
-          <t xml:space="preserve">TRUE</t>
+          <t xml:space="preserve">200</t>
         </is>
       </c>
     </row>
@@ -3669,39 +3664,44 @@
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t xml:space="preserve">Referanse</t>
+          <t xml:space="preserve">Alle navn må stemme</t>
         </is>
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t xml:space="preserve">reference</t>
+          <t xml:space="preserve">requireAllNames</t>
         </is>
       </c>
       <c r="D153" t="inlineStr">
         <is>
-          <t xml:space="preserve">text</t>
+          <t xml:space="preserve">TRUE / FALSE</t>
+        </is>
+      </c>
+      <c r="F153" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TRUE, FALSE</t>
         </is>
       </c>
       <c r="G153" t="inlineStr">
         <is>
-          <t xml:space="preserve">BEP §3.2</t>
+          <t xml:space="preserve">TRUE</t>
         </is>
       </c>
     </row>
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t xml:space="preserve">Etasjer</t>
+          <t xml:space="preserve">Etasjeoppsett</t>
         </is>
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t xml:space="preserve">Navn</t>
+          <t xml:space="preserve">Referanse</t>
         </is>
       </c>
       <c r="C154" t="inlineStr">
         <is>
-          <t xml:space="preserve">storeys.levels[].name</t>
+          <t xml:space="preserve">reference</t>
         </is>
       </c>
       <c r="D154" t="inlineStr">
@@ -3709,14 +3709,9 @@
           <t xml:space="preserve">text</t>
         </is>
       </c>
-      <c r="E154" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
-        </is>
-      </c>
       <c r="G154" t="inlineStr">
         <is>
-          <t xml:space="preserve">Plan 01</t>
+          <t xml:space="preserve">BEP §3.2</t>
         </is>
       </c>
     </row>
@@ -3728,17 +3723,17 @@
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t xml:space="preserve">Kote (m)</t>
+          <t xml:space="preserve">Navn</t>
         </is>
       </c>
       <c r="C155" t="inlineStr">
         <is>
-          <t xml:space="preserve">storeys.levels[].elevation</t>
+          <t xml:space="preserve">storeys.levels[].name</t>
         </is>
       </c>
       <c r="D155" t="inlineStr">
         <is>
-          <t xml:space="preserve">number</t>
+          <t xml:space="preserve">text</t>
         </is>
       </c>
       <c r="E155" t="inlineStr">
@@ -3748,29 +3743,29 @@
       </c>
       <c r="G155" t="inlineStr">
         <is>
-          <t xml:space="preserve">24.15</t>
+          <t xml:space="preserve">Plan 01</t>
         </is>
       </c>
     </row>
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
-          <t xml:space="preserve">Fag</t>
+          <t xml:space="preserve">Etasjer</t>
         </is>
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t xml:space="preserve">Fagkode</t>
+          <t xml:space="preserve">Kote (m)</t>
         </is>
       </c>
       <c r="C156" t="inlineStr">
         <is>
-          <t xml:space="preserve">disciplines[].code</t>
+          <t xml:space="preserve">storeys.levels[].elevation</t>
         </is>
       </c>
       <c r="D156" t="inlineStr">
         <is>
-          <t xml:space="preserve">text</t>
+          <t xml:space="preserve">number</t>
         </is>
       </c>
       <c r="E156" t="inlineStr">
@@ -3780,7 +3775,7 @@
       </c>
       <c r="G156" t="inlineStr">
         <is>
-          <t xml:space="preserve">ARK</t>
+          <t xml:space="preserve">24.15</t>
         </is>
       </c>
     </row>
@@ -3792,17 +3787,17 @@
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t xml:space="preserve">Rapport</t>
+          <t xml:space="preserve">Fagkode</t>
         </is>
       </c>
       <c r="C157" t="inlineStr">
         <is>
-          <t xml:space="preserve">disciplines[].report</t>
+          <t xml:space="preserve">disciplines[].code</t>
         </is>
       </c>
       <c r="D157" t="inlineStr">
         <is>
-          <t xml:space="preserve">TRUE / FALSE</t>
+          <t xml:space="preserve">text</t>
         </is>
       </c>
       <c r="E157" t="inlineStr">
@@ -3810,36 +3805,31 @@
           <t xml:space="preserve">yes</t>
         </is>
       </c>
-      <c r="F157" t="inlineStr">
-        <is>
-          <t xml:space="preserve">TRUE, FALSE</t>
-        </is>
-      </c>
       <c r="G157" t="inlineStr">
         <is>
-          <t xml:space="preserve">TRUE</t>
+          <t xml:space="preserve">ARK</t>
         </is>
       </c>
     </row>
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t xml:space="preserve">Modeller</t>
+          <t xml:space="preserve">Fag</t>
         </is>
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t xml:space="preserve">Modell</t>
+          <t xml:space="preserve">Rapport</t>
         </is>
       </c>
       <c r="C158" t="inlineStr">
         <is>
-          <t xml:space="preserve">models[].label</t>
+          <t xml:space="preserve">disciplines[].report</t>
         </is>
       </c>
       <c r="D158" t="inlineStr">
         <is>
-          <t xml:space="preserve">text</t>
+          <t xml:space="preserve">TRUE / FALSE</t>
         </is>
       </c>
       <c r="E158" t="inlineStr">
@@ -3847,9 +3837,14 @@
           <t xml:space="preserve">yes</t>
         </is>
       </c>
+      <c r="F158" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TRUE, FALSE</t>
+        </is>
+      </c>
       <c r="G158" t="inlineStr">
         <is>
-          <t xml:space="preserve">EKS_ARK</t>
+          <t xml:space="preserve">TRUE</t>
         </is>
       </c>
     </row>
@@ -3861,12 +3856,12 @@
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t xml:space="preserve">Fagkode</t>
+          <t xml:space="preserve">Modell</t>
         </is>
       </c>
       <c r="C159" t="inlineStr">
         <is>
-          <t xml:space="preserve">models[].discipline</t>
+          <t xml:space="preserve">models[].label</t>
         </is>
       </c>
       <c r="D159" t="inlineStr">
@@ -3881,7 +3876,7 @@
       </c>
       <c r="G159" t="inlineStr">
         <is>
-          <t xml:space="preserve">ARK</t>
+          <t xml:space="preserve">EKS_ARK</t>
         </is>
       </c>
     </row>
@@ -3893,17 +3888,22 @@
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t xml:space="preserve">Gruppe</t>
+          <t xml:space="preserve">Fagkode</t>
         </is>
       </c>
       <c r="C160" t="inlineStr">
         <is>
-          <t xml:space="preserve">models[].group</t>
+          <t xml:space="preserve">models[].discipline</t>
         </is>
       </c>
       <c r="D160" t="inlineStr">
         <is>
           <t xml:space="preserve">text</t>
+        </is>
+      </c>
+      <c r="E160" t="inlineStr">
+        <is>
+          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="G160" t="inlineStr">
@@ -3920,22 +3920,22 @@
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t xml:space="preserve">Eierverdier</t>
+          <t xml:space="preserve">Gruppe</t>
         </is>
       </c>
       <c r="C161" t="inlineStr">
         <is>
-          <t xml:space="preserve">models[].ownerNames</t>
+          <t xml:space="preserve">models[].group</t>
         </is>
       </c>
       <c r="D161" t="inlineStr">
         <is>
-          <t xml:space="preserve">list</t>
+          <t xml:space="preserve">text</t>
         </is>
       </c>
       <c r="G161" t="inlineStr">
         <is>
-          <t xml:space="preserve">EKS_ARK, ARK</t>
+          <t xml:space="preserve">ARK</t>
         </is>
       </c>
     </row>
@@ -3947,12 +3947,12 @@
       </c>
       <c r="B162" t="inlineStr">
         <is>
-          <t xml:space="preserve">Gjelder ikke</t>
+          <t xml:space="preserve">Eierverdier</t>
         </is>
       </c>
       <c r="C162" t="inlineStr">
         <is>
-          <t xml:space="preserve">models[].exempt</t>
+          <t xml:space="preserve">models[].ownerNames</t>
         </is>
       </c>
       <c r="D162" t="inlineStr">
@@ -3962,44 +3962,34 @@
       </c>
       <c r="G162" t="inlineStr">
         <is>
-          <t xml:space="preserve">system-classification, phase</t>
+          <t xml:space="preserve">EKS_ARK, ARK</t>
         </is>
       </c>
     </row>
     <row r="163">
       <c r="A163" t="inlineStr">
         <is>
-          <t xml:space="preserve">Standardkrav</t>
+          <t xml:space="preserve">Modeller</t>
         </is>
       </c>
       <c r="B163" t="inlineStr">
         <is>
-          <t xml:space="preserve">Krav</t>
+          <t xml:space="preserve">Gjelder ikke</t>
         </is>
       </c>
       <c r="C163" t="inlineStr">
         <is>
-          <t xml:space="preserve">projectLayer</t>
+          <t xml:space="preserve">models[].exempt</t>
         </is>
       </c>
       <c r="D163" t="inlineStr">
         <is>
-          <t xml:space="preserve">text</t>
-        </is>
-      </c>
-      <c r="E163" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
-        </is>
-      </c>
-      <c r="F163" t="inlineStr">
-        <is>
-          <t xml:space="preserve">ifc-schema, phase, material-product</t>
+          <t xml:space="preserve">list</t>
         </is>
       </c>
       <c r="G163" t="inlineStr">
         <is>
-          <t xml:space="preserve">ifc-schema</t>
+          <t xml:space="preserve">system-classification, phase</t>
         </is>
       </c>
     </row>
@@ -4011,12 +4001,12 @@
       </c>
       <c r="B164" t="inlineStr">
         <is>
-          <t xml:space="preserve">Referanse</t>
+          <t xml:space="preserve">Krav</t>
         </is>
       </c>
       <c r="C164" t="inlineStr">
         <is>
-          <t xml:space="preserve">reference</t>
+          <t xml:space="preserve">projectLayer</t>
         </is>
       </c>
       <c r="D164" t="inlineStr">
@@ -4024,9 +4014,19 @@
           <t xml:space="preserve">text</t>
         </is>
       </c>
+      <c r="E164" t="inlineStr">
+        <is>
+          <t xml:space="preserve">yes</t>
+        </is>
+      </c>
+      <c r="F164" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ifc-schema, phase, material-product</t>
+        </is>
+      </c>
       <c r="G164" t="inlineStr">
         <is>
-          <t xml:space="preserve">BEP §3</t>
+          <t xml:space="preserve">ifc-schema</t>
         </is>
       </c>
     </row>
@@ -4038,22 +4038,22 @@
       </c>
       <c r="B165" t="inlineStr">
         <is>
-          <t xml:space="preserve">Godtatte</t>
+          <t xml:space="preserve">Referanse</t>
         </is>
       </c>
       <c r="C165" t="inlineStr">
         <is>
-          <t xml:space="preserve">accepted</t>
+          <t xml:space="preserve">reference</t>
         </is>
       </c>
       <c r="D165" t="inlineStr">
         <is>
-          <t xml:space="preserve">list</t>
+          <t xml:space="preserve">text</t>
         </is>
       </c>
       <c r="G165" t="inlineStr">
         <is>
-          <t xml:space="preserve">IFC2X3, IFC4</t>
+          <t xml:space="preserve">BEP §3</t>
         </is>
       </c>
     </row>
@@ -4065,12 +4065,12 @@
       </c>
       <c r="B166" t="inlineStr">
         <is>
-          <t xml:space="preserve">Anbefalte</t>
+          <t xml:space="preserve">Godtatte</t>
         </is>
       </c>
       <c r="C166" t="inlineStr">
         <is>
-          <t xml:space="preserve">recommended</t>
+          <t xml:space="preserve">accepted</t>
         </is>
       </c>
       <c r="D166" t="inlineStr">
@@ -4080,44 +4080,34 @@
       </c>
       <c r="G166" t="inlineStr">
         <is>
-          <t xml:space="preserve">IFC4</t>
+          <t xml:space="preserve">IFC2X3, IFC4</t>
         </is>
       </c>
     </row>
     <row r="167">
       <c r="A167" t="inlineStr">
         <is>
-          <t xml:space="preserve">Kilder</t>
+          <t xml:space="preserve">Standardkrav</t>
         </is>
       </c>
       <c r="B167" t="inlineStr">
         <is>
-          <t xml:space="preserve">Krav</t>
+          <t xml:space="preserve">Anbefalte</t>
         </is>
       </c>
       <c r="C167" t="inlineStr">
         <is>
-          <t xml:space="preserve">projectLayer</t>
+          <t xml:space="preserve">recommended</t>
         </is>
       </c>
       <c r="D167" t="inlineStr">
         <is>
-          <t xml:space="preserve">text</t>
-        </is>
-      </c>
-      <c r="E167" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
-        </is>
-      </c>
-      <c r="F167" t="inlineStr">
-        <is>
-          <t xml:space="preserve">phase.sources, material-product.mengdetype, material-product.product, material-product.material</t>
+          <t xml:space="preserve">list</t>
         </is>
       </c>
       <c r="G167" t="inlineStr">
         <is>
-          <t xml:space="preserve">phase.sources</t>
+          <t xml:space="preserve">IFC4</t>
         </is>
       </c>
     </row>
@@ -4129,17 +4119,17 @@
       </c>
       <c r="B168" t="inlineStr">
         <is>
-          <t xml:space="preserve">Kildetype</t>
+          <t xml:space="preserve">Krav</t>
         </is>
       </c>
       <c r="C168" t="inlineStr">
         <is>
-          <t xml:space="preserve">source</t>
+          <t xml:space="preserve">projectLayer</t>
         </is>
       </c>
       <c r="D168" t="inlineStr">
         <is>
-          <t xml:space="preserve">source kind</t>
+          <t xml:space="preserve">text</t>
         </is>
       </c>
       <c r="E168" t="inlineStr">
@@ -4149,12 +4139,12 @@
       </c>
       <c r="F168" t="inlineStr">
         <is>
-          <t xml:space="preserve">attribute, property, classification, material, progressCode</t>
+          <t xml:space="preserve">phase.sources, material-product.mengdetype, material-product.product, material-product.material</t>
         </is>
       </c>
       <c r="G168" t="inlineStr">
         <is>
-          <t xml:space="preserve">property</t>
+          <t xml:space="preserve">phase.sources</t>
         </is>
       </c>
     </row>
@@ -4166,22 +4156,32 @@
       </c>
       <c r="B169" t="inlineStr">
         <is>
-          <t xml:space="preserve">Attributt</t>
+          <t xml:space="preserve">Kildetype</t>
         </is>
       </c>
       <c r="C169" t="inlineStr">
         <is>
-          <t xml:space="preserve">source.attribute</t>
+          <t xml:space="preserve">source</t>
         </is>
       </c>
       <c r="D169" t="inlineStr">
         <is>
-          <t xml:space="preserve">text</t>
+          <t xml:space="preserve">source kind</t>
+        </is>
+      </c>
+      <c r="E169" t="inlineStr">
+        <is>
+          <t xml:space="preserve">yes</t>
+        </is>
+      </c>
+      <c r="F169" t="inlineStr">
+        <is>
+          <t xml:space="preserve">attribute, property, classification, material, progressCode</t>
         </is>
       </c>
       <c r="G169" t="inlineStr">
         <is>
-          <t xml:space="preserve">Name</t>
+          <t xml:space="preserve">property</t>
         </is>
       </c>
     </row>
@@ -4193,12 +4193,12 @@
       </c>
       <c r="B170" t="inlineStr">
         <is>
-          <t xml:space="preserve">Egenskapssett</t>
+          <t xml:space="preserve">Attributt</t>
         </is>
       </c>
       <c r="C170" t="inlineStr">
         <is>
-          <t xml:space="preserve">source.property.propertySet</t>
+          <t xml:space="preserve">source.attribute</t>
         </is>
       </c>
       <c r="D170" t="inlineStr">
@@ -4208,7 +4208,7 @@
       </c>
       <c r="G170" t="inlineStr">
         <is>
-          <t xml:space="preserve">EKS_Project</t>
+          <t xml:space="preserve">Name</t>
         </is>
       </c>
     </row>
@@ -4220,12 +4220,12 @@
       </c>
       <c r="B171" t="inlineStr">
         <is>
-          <t xml:space="preserve">Egenskapsnavn</t>
+          <t xml:space="preserve">Egenskapssett</t>
         </is>
       </c>
       <c r="C171" t="inlineStr">
         <is>
-          <t xml:space="preserve">source.property.name</t>
+          <t xml:space="preserve">source.property.propertySet</t>
         </is>
       </c>
       <c r="D171" t="inlineStr">
@@ -4235,7 +4235,7 @@
       </c>
       <c r="G171" t="inlineStr">
         <is>
-          <t xml:space="preserve">MMI</t>
+          <t xml:space="preserve">EKS_Project</t>
         </is>
       </c>
     </row>
@@ -4247,12 +4247,12 @@
       </c>
       <c r="B172" t="inlineStr">
         <is>
-          <t xml:space="preserve">System</t>
+          <t xml:space="preserve">Egenskapsnavn</t>
         </is>
       </c>
       <c r="C172" t="inlineStr">
         <is>
-          <t xml:space="preserve">source.classification.system</t>
+          <t xml:space="preserve">source.property.name</t>
         </is>
       </c>
       <c r="D172" t="inlineStr">
@@ -4262,37 +4262,64 @@
       </c>
       <c r="G172" t="inlineStr">
         <is>
-          <t xml:space="preserve">NS 3451</t>
+          <t xml:space="preserve">MMI</t>
         </is>
       </c>
     </row>
     <row r="173">
       <c r="A173" t="inlineStr">
         <is>
+          <t xml:space="preserve">Kilder</t>
+        </is>
+      </c>
+      <c r="B173" t="inlineStr">
+        <is>
+          <t xml:space="preserve">System</t>
+        </is>
+      </c>
+      <c r="C173" t="inlineStr">
+        <is>
+          <t xml:space="preserve">source.classification.system</t>
+        </is>
+      </c>
+      <c r="D173" t="inlineStr">
+        <is>
+          <t xml:space="preserve">text</t>
+        </is>
+      </c>
+      <c r="G173" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NS 3451</t>
+        </is>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" t="inlineStr">
+        <is>
           <t xml:space="preserve">Andre regler</t>
         </is>
       </c>
-      <c r="B173" t="inlineStr">
+      <c r="B174" t="inlineStr">
         <is>
           <t xml:space="preserve">Regel</t>
         </is>
       </c>
-      <c r="C173" t="inlineStr">
+      <c r="C174" t="inlineStr">
         <is>
           <t xml:space="preserve">rules[]</t>
         </is>
       </c>
-      <c r="D173" t="inlineStr">
+      <c r="D174" t="inlineStr">
         <is>
           <t xml:space="preserve">JSON</t>
         </is>
       </c>
-      <c r="E173" t="inlineStr">
+      <c r="E174" t="inlineStr">
         <is>
           <t xml:space="preserve">yes</t>
         </is>
       </c>
-      <c r="G173" t="inlineStr">
+      <c r="G174" t="inlineStr">
         <is>
           <t xml:space="preserve">{"id":"elements-typed","kind":"extended","name":"Typed","select":{"entity":{"group":"physicalElement"}},"check":{"type":"element-typed"}}</t>
         </is>
@@ -5464,15 +5491,16 @@
     <col min="5" max="5" width="19" customWidth="1"/>
     <col min="6" max="6" width="20" customWidth="1"/>
     <col min="7" max="7" width="22" customWidth="1"/>
-    <col min="8" max="8" width="22" customWidth="1"/>
-    <col min="9" max="9" width="32" customWidth="1"/>
-    <col min="10" max="10" width="43" customWidth="1"/>
-    <col min="11" max="11" width="36" customWidth="1"/>
-    <col min="12" max="12" width="44" customWidth="1"/>
-    <col min="13" max="13" width="23" customWidth="1"/>
-    <col min="14" max="14" width="17" customWidth="1"/>
-    <col min="15" max="15" width="16" customWidth="1"/>
-    <col min="16" max="16" width="22" customWidth="1"/>
+    <col min="8" max="8" width="24" customWidth="1"/>
+    <col min="9" max="9" width="22" customWidth="1"/>
+    <col min="10" max="10" width="32" customWidth="1"/>
+    <col min="11" max="11" width="43" customWidth="1"/>
+    <col min="12" max="12" width="36" customWidth="1"/>
+    <col min="13" max="13" width="44" customWidth="1"/>
+    <col min="14" max="14" width="23" customWidth="1"/>
+    <col min="15" max="15" width="17" customWidth="1"/>
+    <col min="16" max="16" width="16" customWidth="1"/>
+    <col min="17" max="17" width="22" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -5513,45 +5541,50 @@
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
+          <t xml:space="preserve">Nivå</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
           <t xml:space="preserve">Kildetype</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">Attributt</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">Egenskapssett</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">Egenskapsnavn</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">System</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">Uttrekk (regex)</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">Aktiv</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">Utvalg</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">Instruksjon</t>
         </is>
@@ -5595,45 +5628,50 @@
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
+          <t xml:space="preserve">rules[].check.minLevel</t>
+        </is>
+      </c>
+      <c r="I2" s="2" t="inlineStr">
+        <is>
           <t xml:space="preserve">rules[].check.source</t>
         </is>
       </c>
-      <c r="I2" s="2" t="inlineStr">
+      <c r="J2" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">rules[].check.source.attribute</t>
         </is>
       </c>
-      <c r="J2" s="2" t="inlineStr">
+      <c r="K2" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">rules[].check.source.property.propertySet</t>
         </is>
       </c>
-      <c r="K2" s="2" t="inlineStr">
+      <c r="L2" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">rules[].check.source.property.name</t>
         </is>
       </c>
-      <c r="L2" s="2" t="inlineStr">
+      <c r="M2" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">rules[].check.source.classification.system</t>
         </is>
       </c>
-      <c r="M2" s="2" t="inlineStr">
+      <c r="N2" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">rules[].check.extract</t>
         </is>
       </c>
-      <c r="N2" s="2" t="inlineStr">
+      <c r="O2" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">rules[].enabled</t>
         </is>
       </c>
-      <c r="O2" s="2" t="inlineStr">
+      <c r="P2" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">rules[].select</t>
         </is>
       </c>
-      <c r="P2" s="2" t="inlineStr">
+      <c r="Q2" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">rules[].instructions</t>
         </is>
@@ -5665,27 +5703,27 @@
           <t xml:space="preserve">ns3451</t>
         </is>
       </c>
-      <c r="H3" t="inlineStr">
+      <c r="I3" t="inlineStr">
         <is>
           <t xml:space="preserve">property</t>
         </is>
       </c>
-      <c r="J3" t="inlineStr">
+      <c r="K3" t="inlineStr">
         <is>
           <t xml:space="preserve">&lt;FROM PROJECT&gt;</t>
         </is>
       </c>
-      <c r="K3" t="inlineStr">
+      <c r="L3" t="inlineStr">
         <is>
           <t xml:space="preserve">&lt;FROM PROJECT&gt;</t>
         </is>
       </c>
-      <c r="M3" t="inlineStr">
+      <c r="N3" t="inlineStr">
         <is>
           <t xml:space="preserve">&lt;FROM PROJECT&gt;</t>
         </is>
       </c>
-      <c r="N3" t="b">
+      <c r="O3" t="b">
         <v>1</v>
       </c>
     </row>
@@ -5720,27 +5758,27 @@
           <t xml:space="preserve">occurrence</t>
         </is>
       </c>
-      <c r="H4" t="inlineStr">
+      <c r="I4" t="inlineStr">
         <is>
           <t xml:space="preserve">property</t>
         </is>
       </c>
-      <c r="J4" t="inlineStr">
+      <c r="K4" t="inlineStr">
         <is>
           <t xml:space="preserve">&lt;FROM PROJECT&gt;</t>
         </is>
       </c>
-      <c r="K4" t="inlineStr">
+      <c r="L4" t="inlineStr">
         <is>
           <t xml:space="preserve">&lt;FROM PROJECT&gt;</t>
         </is>
       </c>
-      <c r="M4" t="inlineStr">
+      <c r="N4" t="inlineStr">
         <is>
           <t xml:space="preserve">&lt;FROM PROJECT&gt;</t>
         </is>
       </c>
-      <c r="N4" t="b">
+      <c r="O4" t="b">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Ignore a requirement for the project: Ruleset.ignore, Ignorer in Oppsett
edkjo: "How do I ignore a requirement? Fase isn't a requirement in this
model" ... "per project, not per model". Ruleset.ignore names report row
ids as models[].exempt does; one lookup (notApplicable) serves both, so
every model's row comes back not_applicable with "ignored in the setup
(ignore)" in run, the checks, the report and the board. The config is kept.

Carried through the JSON schema, lint (ignore-unknown warns, duplicate
refused), the workbook (Prosjekt, Ignorert), the config template, and the
IDS export (excluded, code ignored). Oppsett v2: an Ignorer toggle in the
wizard header; an ignored item stays listed, greyed, line 2 Ignorert, the
wizard shows the header alone; its conflicts never hold Lagre.

edkjo, ifc-check/work

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/examples/eks-config-template.xlsx
+++ b/examples/eks-config-template.xlsx
@@ -442,37 +442,42 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
+          <t xml:space="preserve">Requirement that does not apply to the project</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Prosjekt</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ignorert (requirement ids, as Gjelder ikke)</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
           <t xml:space="preserve">Every element typed, unique attribute, type used N times, header or unit fact</t>
         </is>
       </c>
-      <c r="B26" t="inlineStr">
+      <c r="B27" t="inlineStr">
         <is>
           <t xml:space="preserve">Andre regler</t>
         </is>
       </c>
-      <c r="C26" t="inlineStr">
+      <c r="C27" t="inlineStr">
         <is>
           <t xml:space="preserve">one JSON rule per row (docs: AGENTS.md Rulesets)</t>
         </is>
       </c>
     </row>
-    <row r="27"/>
-    <row r="28">
-      <c r="A28" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Conventions</t>
-        </is>
-      </c>
-    </row>
+    <row r="28"/>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
-        </is>
-      </c>
-      <c r="B29" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Row 1 is the label, row 2 the field path, data from row 3. Never edit row 2. Columns may move. A column with a blank row 2 is a note, never read.</t>
+          <t xml:space="preserve">Conventions</t>
         </is>
       </c>
     </row>
@@ -484,7 +489,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t xml:space="preserve">Replace every &lt;FROM PROJECT&gt;. Lint refuses the file while one remains.</t>
+          <t xml:space="preserve">Row 1 is the label, row 2 the field path, data from row 3. Never edit row 2. Columns may move. A column with a blank row 2 is a note, never read.</t>
         </is>
       </c>
     </row>
@@ -496,7 +501,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t xml:space="preserve">No evidence in the BEP, EIR or manual for a row: delete the row. Never copy a value from a model as the requirement.</t>
+          <t xml:space="preserve">Replace every &lt;FROM PROJECT&gt;. Lint refuses the file while one remains.</t>
         </is>
       </c>
     </row>
@@ -508,7 +513,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t xml:space="preserve">A row with only key cells filled (Krav, Rolle, ID, Aktiv, Rapport) is not declared and is dropped. A row with a value and a blank required cell is refused at that cell.</t>
+          <t xml:space="preserve">No evidence in the BEP, EIR or manual for a row: delete the row. Never copy a value from a model as the requirement.</t>
         </is>
       </c>
     </row>
@@ -520,7 +525,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t xml:space="preserve">Aktiv, Rapport and Alle navn må stemme take TRUE or FALSE. Blank is refused. Aktiv FALSE keeps the rule and switches it off.</t>
+          <t xml:space="preserve">A row with only key cells filled (Krav, Rolle, ID, Aktiv, Rapport) is not declared and is dropped. A row with a value and a blank required cell is refused at that cell.</t>
         </is>
       </c>
     </row>
@@ -532,7 +537,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t xml:space="preserve">Lists are comma-separated. A value containing a comma cannot be written in a list.</t>
+          <t xml:space="preserve">Aktiv, Rapport and Alle navn må stemme take TRUE or FALSE. Blank is refused. Aktiv FALSE keeps the rule and switches it off.</t>
         </is>
       </c>
     </row>
@@ -544,7 +549,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t xml:space="preserve">Rule IDs are unique across IDS, Klassifikasjon, MMI, Kopiobjekt and Andre regler.</t>
+          <t xml:space="preserve">Lists are comma-separated. A value containing a comma cannot be written in a list.</t>
         </is>
       </c>
     </row>
@@ -556,7 +561,7 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t xml:space="preserve">Referanse is the citation (BEP §3.2). Beskrivelse says what the rule checks.</t>
+          <t xml:space="preserve">Rule IDs are unique across IDS, Klassifikasjon, MMI, Kopiobjekt and Andre regler.</t>
         </is>
       </c>
     </row>
@@ -568,7 +573,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t xml:space="preserve">Kote is metres, measured to Referanseplan: OKFG (OK ferdig gulv) or OKBD (OK bærende dekke).</t>
+          <t xml:space="preserve">Referanse is the citation (BEP §3.2). Beskrivelse says what the rule checks.</t>
         </is>
       </c>
     </row>
@@ -580,7 +585,7 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t xml:space="preserve">Tolerances and windows are millimetres, file minus level. Blank = no limit. 0 = exact.</t>
+          <t xml:space="preserve">Kote is metres, measured to Referanseplan: OKFG (OK ferdig gulv) or OKBD (OK bærende dekke).</t>
         </is>
       </c>
     </row>
@@ -592,7 +597,7 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t xml:space="preserve">Etasjeoppsett: one row with Fagkode blank for the project. One more row per discipline measuring to another plane, with Alle navn må stemme.</t>
+          <t xml:space="preserve">Tolerances and windows are millimetres, file minus level. Blank = no limit. 0 = exact.</t>
         </is>
       </c>
     </row>
@@ -604,7 +609,7 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t xml:space="preserve">Modell is the IFC file name without extension, exact (EKS_ARK for EKS_ARK.ifc).</t>
+          <t xml:space="preserve">Etasjeoppsett: one row with Fagkode blank for the project. One more row per discipline measuring to another plane, with Alle navn må stemme.</t>
         </is>
       </c>
     </row>
@@ -616,7 +621,7 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t xml:space="preserve">Kopiobjekt: compared ignoring case and whitespace. Blank, an own value or this model's Eierverdier = the file's own object. A copy value or any other value = a copy.</t>
+          <t xml:space="preserve">Modell is the IFC file name without extension, exact (EKS_ARK for EKS_ARK.ifc).</t>
         </is>
       </c>
     </row>
@@ -628,7 +633,7 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t xml:space="preserve">Kildetype: attribute, property, classification, material, progressCode. material only in the rule sheets. Never material under material-product.material: IfcRelAssociatesMaterial is read first already. progressCode only under phase.sources.</t>
+          <t xml:space="preserve">Kopiobjekt: compared ignoring case and whitespace. Blank, an own value or this model's Eierverdier = the file's own object. A copy value or any other value = a copy.</t>
         </is>
       </c>
     </row>
@@ -640,7 +645,7 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t xml:space="preserve">Uttrekk is a JavaScript regex with exactly one capture group: the code.</t>
+          <t xml:space="preserve">Kildetype: attribute, property, classification, material, progressCode. material only in the rule sheets. Never material under material-product.material: IfcRelAssociatesMaterial is read first already. progressCode only under phase.sources.</t>
         </is>
       </c>
     </row>
@@ -652,7 +657,7 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t xml:space="preserve">IDS-fasetter: Spesifikasjon names an IDS row's ID. Del is applicability or requirements. Kardinalitet only under requirements; partOf takes required or prohibited.</t>
+          <t xml:space="preserve">Uttrekk is a JavaScript regex with exactly one capture group: the code.</t>
         </is>
       </c>
     </row>
@@ -664,7 +669,7 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t xml:space="preserve">IDS-fasetter: a value is Verdi, or a restriction (Grunntype, Verdiliste, Mønster, Min, Maks, Over, Under, Lengde, Min lengde, Maks lengde). A non-empty value is Min lengde 1. Names (Attributt, Egenskapssett, Egenskap, System) are literal.</t>
+          <t xml:space="preserve">IDS-fasetter: Spesifikasjon names an IDS row's ID. Del is applicability or requirements. Kardinalitet only under requirements; partOf takes required or prohibited.</t>
         </is>
       </c>
     </row>
@@ -676,7 +681,7 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t xml:space="preserve">IFC-klasse: concrete classes, uppercase (IFCWALL). An abstract class matches nothing: use Klassegruppe.</t>
+          <t xml:space="preserve">IDS-fasetter: a value is Verdi, or a restriction (Grunntype, Verdiliste, Mønster, Min, Maks, Over, Under, Lengde, Min lengde, Maks lengde). A non-empty value is Min lengde 1. Names (Attributt, Egenskapssett, Egenskap, System) are literal.</t>
         </is>
       </c>
     </row>
@@ -688,82 +693,57 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
+          <t xml:space="preserve">IFC-klasse: concrete classes, uppercase (IFCWALL). An abstract class matches nothing: use Klassegruppe.</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
           <t xml:space="preserve">Gjelder ikke takes requirement ids: parse-integrity, spatial-chain, storey-containment, storey-in-building, storey-elevation, guid-unique, element-named, element-typed, type-name-placeholder, single-instance-types, type-unused, element-material, storey-config, mesh-placement, body-no-mesh, ifc-schema, phase, material-product, system-classification, component-classification, progress-code, copy-object, tfm, type-name, or an Andre regler rule ID.</t>
         </is>
       </c>
     </row>
-    <row r="48"/>
-    <row r="49">
-      <c r="A49" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Sheet</t>
-        </is>
-      </c>
-      <c r="B49" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Column</t>
-        </is>
-      </c>
-      <c r="C49" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Field</t>
-        </is>
-      </c>
-      <c r="D49" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Type</t>
-        </is>
-      </c>
-      <c r="E49" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Required</t>
-        </is>
-      </c>
-      <c r="F49" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Allowed</t>
-        </is>
-      </c>
-      <c r="G49" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Example</t>
-        </is>
-      </c>
-    </row>
+    <row r="49"/>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t xml:space="preserve">Prosjekt</t>
+          <t xml:space="preserve">Sheet</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t xml:space="preserve">Formatversjon</t>
+          <t xml:space="preserve">Column</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t xml:space="preserve">formatVersion</t>
+          <t xml:space="preserve">Field</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t xml:space="preserve">number</t>
+          <t xml:space="preserve">Type</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t xml:space="preserve">yes</t>
+          <t xml:space="preserve">Required</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t xml:space="preserve">2</t>
+          <t xml:space="preserve">Allowed</t>
         </is>
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t xml:space="preserve">2</t>
+          <t xml:space="preserve">Example</t>
         </is>
       </c>
     </row>
@@ -775,17 +755,17 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t xml:space="preserve">Navn</t>
+          <t xml:space="preserve">Formatversjon</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t xml:space="preserve">name</t>
+          <t xml:space="preserve">formatVersion</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t xml:space="preserve">text</t>
+          <t xml:space="preserve">number</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
@@ -793,9 +773,14 @@
           <t xml:space="preserve">yes</t>
         </is>
       </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2</t>
+        </is>
+      </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t xml:space="preserve">EKS</t>
+          <t xml:space="preserve">2</t>
         </is>
       </c>
     </row>
@@ -807,12 +792,12 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t xml:space="preserve">Beskrivelse</t>
+          <t xml:space="preserve">Navn</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t xml:space="preserve">description</t>
+          <t xml:space="preserve">name</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
@@ -820,9 +805,14 @@
           <t xml:space="preserve">text</t>
         </is>
       </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t xml:space="preserve">yes</t>
+        </is>
+      </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t xml:space="preserve">BEP 2.0</t>
+          <t xml:space="preserve">EKS</t>
         </is>
       </c>
     </row>
@@ -834,32 +824,22 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t xml:space="preserve">IFC-versjoner</t>
+          <t xml:space="preserve">Beskrivelse</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t xml:space="preserve">ifcVersions</t>
+          <t xml:space="preserve">description</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t xml:space="preserve">list</t>
-        </is>
-      </c>
-      <c r="E53" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
-        </is>
-      </c>
-      <c r="F53" t="inlineStr">
-        <is>
-          <t xml:space="preserve">IFC2X3, IFC4, IFC4X3_ADD2</t>
+          <t xml:space="preserve">text</t>
         </is>
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t xml:space="preserve">IFC2X3, IFC4</t>
+          <t xml:space="preserve">BEP 2.0</t>
         </is>
       </c>
     </row>
@@ -871,17 +851,32 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t xml:space="preserve">Tittel</t>
+          <t xml:space="preserve">IFC-versjoner</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t xml:space="preserve">info.title</t>
+          <t xml:space="preserve">ifcVersions</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t xml:space="preserve">text</t>
+          <t xml:space="preserve">list</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">yes</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">IFC2X3, IFC4, IFC4X3_ADD2</t>
+        </is>
+      </c>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">IFC2X3, IFC4</t>
         </is>
       </c>
     </row>
@@ -893,22 +888,22 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t xml:space="preserve">Versjon</t>
+          <t xml:space="preserve">Ignorert</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t xml:space="preserve">info.version</t>
+          <t xml:space="preserve">ignore</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t xml:space="preserve">text</t>
+          <t xml:space="preserve">list</t>
         </is>
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t xml:space="preserve">1.0</t>
+          <t xml:space="preserve">phase</t>
         </is>
       </c>
     </row>
@@ -920,12 +915,12 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t xml:space="preserve">IDS-beskrivelse</t>
+          <t xml:space="preserve">Tittel</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t xml:space="preserve">info.description</t>
+          <t xml:space="preserve">info.title</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
@@ -942,12 +937,12 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t xml:space="preserve">Forfatter</t>
+          <t xml:space="preserve">Versjon</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t xml:space="preserve">info.author</t>
+          <t xml:space="preserve">info.version</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
@@ -957,7 +952,7 @@
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t xml:space="preserve">post@example.no</t>
+          <t xml:space="preserve">1.0</t>
         </is>
       </c>
     </row>
@@ -969,22 +964,17 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t xml:space="preserve">Dato</t>
+          <t xml:space="preserve">IDS-beskrivelse</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t xml:space="preserve">info.date</t>
+          <t xml:space="preserve">info.description</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
           <t xml:space="preserve">text</t>
-        </is>
-      </c>
-      <c r="G58" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2026-09-29</t>
         </is>
       </c>
     </row>
@@ -996,17 +986,22 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t xml:space="preserve">Formål</t>
+          <t xml:space="preserve">Forfatter</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t xml:space="preserve">info.purpose</t>
+          <t xml:space="preserve">info.author</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
           <t xml:space="preserve">text</t>
+        </is>
+      </c>
+      <c r="G59" t="inlineStr">
+        <is>
+          <t xml:space="preserve">post@example.no</t>
         </is>
       </c>
     </row>
@@ -1018,17 +1013,22 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t xml:space="preserve">Milepæl</t>
+          <t xml:space="preserve">Dato</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t xml:space="preserve">info.milestone</t>
+          <t xml:space="preserve">info.date</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
           <t xml:space="preserve">text</t>
+        </is>
+      </c>
+      <c r="G60" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-29</t>
         </is>
       </c>
     </row>
@@ -1040,12 +1040,12 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t xml:space="preserve">Opphavsrett</t>
+          <t xml:space="preserve">Formål</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t xml:space="preserve">info.copyright</t>
+          <t xml:space="preserve">info.purpose</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
@@ -1062,12 +1062,12 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t xml:space="preserve">JSON-skjema</t>
+          <t xml:space="preserve">Milepæl</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t xml:space="preserve">$schema</t>
+          <t xml:space="preserve">info.milestone</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
@@ -1079,64 +1079,44 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t xml:space="preserve">IDS</t>
+          <t xml:space="preserve">Prosjekt</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t xml:space="preserve">ID</t>
+          <t xml:space="preserve">Opphavsrett</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t xml:space="preserve">rules[].id</t>
+          <t xml:space="preserve">info.copyright</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
           <t xml:space="preserve">text</t>
-        </is>
-      </c>
-      <c r="E63" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
-        </is>
-      </c>
-      <c r="G63" t="inlineStr">
-        <is>
-          <t xml:space="preserve">eks-material</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t xml:space="preserve">IDS</t>
+          <t xml:space="preserve">Prosjekt</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t xml:space="preserve">Navn</t>
+          <t xml:space="preserve">JSON-skjema</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t xml:space="preserve">rules[].name</t>
+          <t xml:space="preserve">$schema</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
           <t xml:space="preserve">text</t>
-        </is>
-      </c>
-      <c r="E64" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
-        </is>
-      </c>
-      <c r="G64" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Physical elements carry a material</t>
         </is>
       </c>
     </row>
@@ -1148,17 +1128,27 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t xml:space="preserve">Beskrivelse</t>
+          <t xml:space="preserve">ID</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t xml:space="preserve">rules[].description</t>
+          <t xml:space="preserve">rules[].id</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
           <t xml:space="preserve">text</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t xml:space="preserve">yes</t>
+        </is>
+      </c>
+      <c r="G65" t="inlineStr">
+        <is>
+          <t xml:space="preserve">eks-material</t>
         </is>
       </c>
     </row>
@@ -1170,12 +1160,12 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t xml:space="preserve">Referanse</t>
+          <t xml:space="preserve">Navn</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t xml:space="preserve">rules[].reference</t>
+          <t xml:space="preserve">rules[].name</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
@@ -1183,9 +1173,14 @@
           <t xml:space="preserve">text</t>
         </is>
       </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t xml:space="preserve">yes</t>
+        </is>
+      </c>
       <c r="G66" t="inlineStr">
         <is>
-          <t xml:space="preserve">BEP §6.12</t>
+          <t xml:space="preserve">Physical elements carry a material</t>
         </is>
       </c>
     </row>
@@ -1197,12 +1192,12 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t xml:space="preserve">Instruksjon</t>
+          <t xml:space="preserve">Beskrivelse</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t xml:space="preserve">rules[].instructions</t>
+          <t xml:space="preserve">rules[].description</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
@@ -1219,17 +1214,22 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t xml:space="preserve">Identifikator</t>
+          <t xml:space="preserve">Referanse</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t xml:space="preserve">rules[].identifier</t>
+          <t xml:space="preserve">rules[].reference</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
         <is>
           <t xml:space="preserve">text</t>
+        </is>
+      </c>
+      <c r="G68" t="inlineStr">
+        <is>
+          <t xml:space="preserve">BEP §6.12</t>
         </is>
       </c>
     </row>
@@ -1241,22 +1241,17 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t xml:space="preserve">IFC-versjoner</t>
+          <t xml:space="preserve">Instruksjon</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t xml:space="preserve">rules[].ifcVersions</t>
+          <t xml:space="preserve">rules[].instructions</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t xml:space="preserve">list</t>
-        </is>
-      </c>
-      <c r="F69" t="inlineStr">
-        <is>
-          <t xml:space="preserve">IFC2X3, IFC4, IFC4X3_ADD2</t>
+          <t xml:space="preserve">text</t>
         </is>
       </c>
     </row>
@@ -1268,22 +1263,17 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t xml:space="preserve">Min forekomster</t>
+          <t xml:space="preserve">Identifikator</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t xml:space="preserve">rules[].applicability.minOccurs</t>
+          <t xml:space="preserve">rules[].identifier</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t xml:space="preserve">number</t>
-        </is>
-      </c>
-      <c r="G70" t="inlineStr">
-        <is>
-          <t xml:space="preserve">1</t>
+          <t xml:space="preserve">text</t>
         </is>
       </c>
     </row>
@@ -1295,22 +1285,22 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t xml:space="preserve">Maks forekomster</t>
+          <t xml:space="preserve">IFC-versjoner</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t xml:space="preserve">rules[].applicability.maxOccurs</t>
+          <t xml:space="preserve">rules[].ifcVersions</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t xml:space="preserve">whole number or unbounded</t>
-        </is>
-      </c>
-      <c r="G71" t="inlineStr">
-        <is>
-          <t xml:space="preserve">unbounded</t>
+          <t xml:space="preserve">list</t>
+        </is>
+      </c>
+      <c r="F71" t="inlineStr">
+        <is>
+          <t xml:space="preserve">IFC2X3, IFC4, IFC4X3_ADD2</t>
         </is>
       </c>
     </row>
@@ -1322,17 +1312,22 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t xml:space="preserve">Kravbeskrivelse</t>
+          <t xml:space="preserve">Min forekomster</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t xml:space="preserve">rules[].requirements.description</t>
+          <t xml:space="preserve">rules[].applicability.minOccurs</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t xml:space="preserve">text</t>
+          <t xml:space="preserve">number</t>
+        </is>
+      </c>
+      <c r="G72" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1</t>
         </is>
       </c>
     </row>
@@ -1344,86 +1339,66 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t xml:space="preserve">Aktiv</t>
+          <t xml:space="preserve">Maks forekomster</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t xml:space="preserve">rules[].enabled</t>
+          <t xml:space="preserve">rules[].applicability.maxOccurs</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t xml:space="preserve">TRUE / FALSE</t>
-        </is>
-      </c>
-      <c r="E73" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
-        </is>
-      </c>
-      <c r="F73" t="inlineStr">
-        <is>
-          <t xml:space="preserve">TRUE, FALSE</t>
+          <t xml:space="preserve">whole number or unbounded</t>
         </is>
       </c>
       <c r="G73" t="inlineStr">
         <is>
-          <t xml:space="preserve">TRUE</t>
+          <t xml:space="preserve">unbounded</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t xml:space="preserve">IDS-fasetter</t>
+          <t xml:space="preserve">IDS</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t xml:space="preserve">Spesifikasjon</t>
+          <t xml:space="preserve">Kravbeskrivelse</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t xml:space="preserve">spec</t>
+          <t xml:space="preserve">rules[].requirements.description</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
         <is>
           <t xml:space="preserve">text</t>
-        </is>
-      </c>
-      <c r="E74" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
-        </is>
-      </c>
-      <c r="G74" t="inlineStr">
-        <is>
-          <t xml:space="preserve">eks-material</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t xml:space="preserve">IDS-fasetter</t>
+          <t xml:space="preserve">IDS</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t xml:space="preserve">Del</t>
+          <t xml:space="preserve">Aktiv</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t xml:space="preserve">part</t>
+          <t xml:space="preserve">rules[].enabled</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t xml:space="preserve">text</t>
+          <t xml:space="preserve">TRUE / FALSE</t>
         </is>
       </c>
       <c r="E75" t="inlineStr">
@@ -1433,12 +1408,12 @@
       </c>
       <c r="F75" t="inlineStr">
         <is>
-          <t xml:space="preserve">applicability, requirements</t>
+          <t xml:space="preserve">TRUE, FALSE</t>
         </is>
       </c>
       <c r="G75" t="inlineStr">
         <is>
-          <t xml:space="preserve">requirements</t>
+          <t xml:space="preserve">TRUE</t>
         </is>
       </c>
     </row>
@@ -1450,12 +1425,12 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t xml:space="preserve">Fasett</t>
+          <t xml:space="preserve">Spesifikasjon</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t xml:space="preserve">facet</t>
+          <t xml:space="preserve">spec</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
@@ -1468,14 +1443,9 @@
           <t xml:space="preserve">yes</t>
         </is>
       </c>
-      <c r="F76" t="inlineStr">
-        <is>
-          <t xml:space="preserve">entity, partOf, classification, attribute, property, material</t>
-        </is>
-      </c>
       <c r="G76" t="inlineStr">
         <is>
-          <t xml:space="preserve">material</t>
+          <t xml:space="preserve">eks-material</t>
         </is>
       </c>
     </row>
@@ -1487,22 +1457,32 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t xml:space="preserve">IFC-klasse</t>
+          <t xml:space="preserve">Del</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t xml:space="preserve">classes</t>
+          <t xml:space="preserve">part</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t xml:space="preserve">list</t>
+          <t xml:space="preserve">text</t>
+        </is>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t xml:space="preserve">yes</t>
+        </is>
+      </c>
+      <c r="F77" t="inlineStr">
+        <is>
+          <t xml:space="preserve">applicability, requirements</t>
         </is>
       </c>
       <c r="G77" t="inlineStr">
         <is>
-          <t xml:space="preserve">IFCWALL, IFCSLAB</t>
+          <t xml:space="preserve">requirements</t>
         </is>
       </c>
     </row>
@@ -1514,12 +1494,12 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t xml:space="preserve">Klassegruppe</t>
+          <t xml:space="preserve">Fasett</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t xml:space="preserve">group</t>
+          <t xml:space="preserve">facet</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
@@ -1527,14 +1507,19 @@
           <t xml:space="preserve">text</t>
         </is>
       </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t xml:space="preserve">yes</t>
+        </is>
+      </c>
       <c r="F78" t="inlineStr">
         <is>
-          <t xml:space="preserve">product, element, physicalElement, builtElement, distributionElement, spatialElement, featureElement, elementType, typeProduct, group</t>
+          <t xml:space="preserve">entity, partOf, classification, attribute, property, material</t>
         </is>
       </c>
       <c r="G78" t="inlineStr">
         <is>
-          <t xml:space="preserve">physicalElement</t>
+          <t xml:space="preserve">material</t>
         </is>
       </c>
     </row>
@@ -1546,22 +1531,22 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t xml:space="preserve">PredefinedType</t>
+          <t xml:space="preserve">IFC-klasse</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t xml:space="preserve">predefinedType</t>
+          <t xml:space="preserve">classes</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t xml:space="preserve">text</t>
+          <t xml:space="preserve">list</t>
         </is>
       </c>
       <c r="G79" t="inlineStr">
         <is>
-          <t xml:space="preserve">SOLIDWALL</t>
+          <t xml:space="preserve">IFCWALL, IFCSLAB</t>
         </is>
       </c>
     </row>
@@ -1573,12 +1558,12 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t xml:space="preserve">Attributt</t>
+          <t xml:space="preserve">Klassegruppe</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t xml:space="preserve">name</t>
+          <t xml:space="preserve">group</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
@@ -1586,9 +1571,14 @@
           <t xml:space="preserve">text</t>
         </is>
       </c>
+      <c r="F80" t="inlineStr">
+        <is>
+          <t xml:space="preserve">product, element, physicalElement, builtElement, distributionElement, spatialElement, featureElement, elementType, typeProduct, group</t>
+        </is>
+      </c>
       <c r="G80" t="inlineStr">
         <is>
-          <t xml:space="preserve">Name</t>
+          <t xml:space="preserve">physicalElement</t>
         </is>
       </c>
     </row>
@@ -1600,12 +1590,12 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t xml:space="preserve">Egenskapssett</t>
+          <t xml:space="preserve">PredefinedType</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t xml:space="preserve">propertySet</t>
+          <t xml:space="preserve">predefinedType</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
@@ -1615,7 +1605,7 @@
       </c>
       <c r="G81" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pset_WallCommon</t>
+          <t xml:space="preserve">SOLIDWALL</t>
         </is>
       </c>
     </row>
@@ -1627,12 +1617,12 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t xml:space="preserve">Egenskapsnavn</t>
+          <t xml:space="preserve">Attributt</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t xml:space="preserve">baseName</t>
+          <t xml:space="preserve">name</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
@@ -1642,7 +1632,7 @@
       </c>
       <c r="G82" t="inlineStr">
         <is>
-          <t xml:space="preserve">FireRating</t>
+          <t xml:space="preserve">Name</t>
         </is>
       </c>
     </row>
@@ -1654,12 +1644,12 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t xml:space="preserve">Datatype</t>
+          <t xml:space="preserve">Egenskapssett</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t xml:space="preserve">dataType</t>
+          <t xml:space="preserve">propertySet</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
@@ -1669,7 +1659,7 @@
       </c>
       <c r="G83" t="inlineStr">
         <is>
-          <t xml:space="preserve">IFCLABEL</t>
+          <t xml:space="preserve">Pset_WallCommon</t>
         </is>
       </c>
     </row>
@@ -1681,12 +1671,12 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t xml:space="preserve">System</t>
+          <t xml:space="preserve">Egenskapsnavn</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t xml:space="preserve">system</t>
+          <t xml:space="preserve">baseName</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
@@ -1696,7 +1686,7 @@
       </c>
       <c r="G84" t="inlineStr">
         <is>
-          <t xml:space="preserve">NS 3451</t>
+          <t xml:space="preserve">FireRating</t>
         </is>
       </c>
     </row>
@@ -1708,12 +1698,12 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t xml:space="preserve">Relasjon</t>
+          <t xml:space="preserve">Datatype</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t xml:space="preserve">relation</t>
+          <t xml:space="preserve">dataType</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
@@ -1721,14 +1711,9 @@
           <t xml:space="preserve">text</t>
         </is>
       </c>
-      <c r="F85" t="inlineStr">
-        <is>
-          <t xml:space="preserve">IFCRELAGGREGATES, IFCRELASSIGNSTOGROUP, IFCRELCONTAINEDINSPATIALSTRUCTURE, IFCRELNESTS, IFCRELVOIDSELEMENT IFCRELFILLSELEMENT</t>
-        </is>
-      </c>
       <c r="G85" t="inlineStr">
         <is>
-          <t xml:space="preserve">IFCRELCONTAINEDINSPATIALSTRUCTURE</t>
+          <t xml:space="preserve">IFCLABEL</t>
         </is>
       </c>
     </row>
@@ -1740,12 +1725,12 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t xml:space="preserve">Verdi</t>
+          <t xml:space="preserve">System</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t xml:space="preserve">value</t>
+          <t xml:space="preserve">system</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
@@ -1755,7 +1740,7 @@
       </c>
       <c r="G86" t="inlineStr">
         <is>
-          <t xml:space="preserve">EI 60</t>
+          <t xml:space="preserve">NS 3451</t>
         </is>
       </c>
     </row>
@@ -1767,22 +1752,27 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t xml:space="preserve">Verdiliste</t>
+          <t xml:space="preserve">Relasjon</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t xml:space="preserve">value.enumeration</t>
+          <t xml:space="preserve">relation</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t xml:space="preserve">list</t>
+          <t xml:space="preserve">text</t>
+        </is>
+      </c>
+      <c r="F87" t="inlineStr">
+        <is>
+          <t xml:space="preserve">IFCRELAGGREGATES, IFCRELASSIGNSTOGROUP, IFCRELCONTAINEDINSPATIALSTRUCTURE, IFCRELNESTS, IFCRELVOIDSELEMENT IFCRELFILLSELEMENT</t>
         </is>
       </c>
       <c r="G87" t="inlineStr">
         <is>
-          <t xml:space="preserve">EI 30, EI 60</t>
+          <t xml:space="preserve">IFCRELCONTAINEDINSPATIALSTRUCTURE</t>
         </is>
       </c>
     </row>
@@ -1794,12 +1784,12 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t xml:space="preserve">Mønster</t>
+          <t xml:space="preserve">Verdi</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t xml:space="preserve">value.pattern</t>
+          <t xml:space="preserve">value</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
@@ -1809,7 +1799,7 @@
       </c>
       <c r="G88" t="inlineStr">
         <is>
-          <t xml:space="preserve">EI \d+</t>
+          <t xml:space="preserve">EI 60</t>
         </is>
       </c>
     </row>
@@ -1821,27 +1811,22 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t xml:space="preserve">Grunntype</t>
+          <t xml:space="preserve">Verdiliste</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t xml:space="preserve">value.base</t>
+          <t xml:space="preserve">value.enumeration</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t xml:space="preserve">text</t>
-        </is>
-      </c>
-      <c r="F89" t="inlineStr">
-        <is>
-          <t xml:space="preserve">string, boolean, integer, double, decimal, date, dateTime, duration</t>
+          <t xml:space="preserve">list</t>
         </is>
       </c>
       <c r="G89" t="inlineStr">
         <is>
-          <t xml:space="preserve">double</t>
+          <t xml:space="preserve">EI 30, EI 60</t>
         </is>
       </c>
     </row>
@@ -1853,22 +1838,22 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t xml:space="preserve">Min</t>
+          <t xml:space="preserve">Mønster</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t xml:space="preserve">value.minInclusive</t>
+          <t xml:space="preserve">value.pattern</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t xml:space="preserve">number</t>
+          <t xml:space="preserve">text</t>
         </is>
       </c>
       <c r="G90" t="inlineStr">
         <is>
-          <t xml:space="preserve">0</t>
+          <t xml:space="preserve">EI \d+</t>
         </is>
       </c>
     </row>
@@ -1880,22 +1865,27 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t xml:space="preserve">Maks</t>
+          <t xml:space="preserve">Grunntype</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t xml:space="preserve">value.maxInclusive</t>
+          <t xml:space="preserve">value.base</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t xml:space="preserve">number</t>
+          <t xml:space="preserve">text</t>
+        </is>
+      </c>
+      <c r="F91" t="inlineStr">
+        <is>
+          <t xml:space="preserve">string, boolean, integer, double, decimal, date, dateTime, duration</t>
         </is>
       </c>
       <c r="G91" t="inlineStr">
         <is>
-          <t xml:space="preserve">100</t>
+          <t xml:space="preserve">double</t>
         </is>
       </c>
     </row>
@@ -1907,12 +1897,12 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t xml:space="preserve">Over</t>
+          <t xml:space="preserve">Min</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t xml:space="preserve">value.minExclusive</t>
+          <t xml:space="preserve">value.minInclusive</t>
         </is>
       </c>
       <c r="D92" t="inlineStr">
@@ -1934,12 +1924,12 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t xml:space="preserve">Under</t>
+          <t xml:space="preserve">Maks</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t xml:space="preserve">value.maxExclusive</t>
+          <t xml:space="preserve">value.maxInclusive</t>
         </is>
       </c>
       <c r="D93" t="inlineStr">
@@ -1961,12 +1951,12 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t xml:space="preserve">Lengde</t>
+          <t xml:space="preserve">Over</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t xml:space="preserve">value.length</t>
+          <t xml:space="preserve">value.minExclusive</t>
         </is>
       </c>
       <c r="D94" t="inlineStr">
@@ -1976,7 +1966,7 @@
       </c>
       <c r="G94" t="inlineStr">
         <is>
-          <t xml:space="preserve">3</t>
+          <t xml:space="preserve">0</t>
         </is>
       </c>
     </row>
@@ -1988,12 +1978,12 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t xml:space="preserve">Min lengde</t>
+          <t xml:space="preserve">Under</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t xml:space="preserve">value.minLength</t>
+          <t xml:space="preserve">value.maxExclusive</t>
         </is>
       </c>
       <c r="D95" t="inlineStr">
@@ -2003,7 +1993,7 @@
       </c>
       <c r="G95" t="inlineStr">
         <is>
-          <t xml:space="preserve">1</t>
+          <t xml:space="preserve">100</t>
         </is>
       </c>
     </row>
@@ -2015,12 +2005,12 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t xml:space="preserve">Maks lengde</t>
+          <t xml:space="preserve">Lengde</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t xml:space="preserve">value.maxLength</t>
+          <t xml:space="preserve">value.length</t>
         </is>
       </c>
       <c r="D96" t="inlineStr">
@@ -2030,7 +2020,7 @@
       </c>
       <c r="G96" t="inlineStr">
         <is>
-          <t xml:space="preserve">20</t>
+          <t xml:space="preserve">3</t>
         </is>
       </c>
     </row>
@@ -2042,17 +2032,22 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t xml:space="preserve">URI</t>
+          <t xml:space="preserve">Min lengde</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t xml:space="preserve">uri</t>
+          <t xml:space="preserve">value.minLength</t>
         </is>
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t xml:space="preserve">text</t>
+          <t xml:space="preserve">number</t>
+        </is>
+      </c>
+      <c r="G97" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1</t>
         </is>
       </c>
     </row>
@@ -2064,27 +2059,22 @@
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t xml:space="preserve">Kardinalitet</t>
+          <t xml:space="preserve">Maks lengde</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t xml:space="preserve">cardinality</t>
+          <t xml:space="preserve">value.maxLength</t>
         </is>
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t xml:space="preserve">text</t>
-        </is>
-      </c>
-      <c r="F98" t="inlineStr">
-        <is>
-          <t xml:space="preserve">required, optional, prohibited</t>
+          <t xml:space="preserve">number</t>
         </is>
       </c>
       <c r="G98" t="inlineStr">
         <is>
-          <t xml:space="preserve">required</t>
+          <t xml:space="preserve">20</t>
         </is>
       </c>
     </row>
@@ -2096,12 +2086,12 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t xml:space="preserve">Instruksjon</t>
+          <t xml:space="preserve">URI</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t xml:space="preserve">instructions</t>
+          <t xml:space="preserve">uri</t>
         </is>
       </c>
       <c r="D99" t="inlineStr">
@@ -2113,17 +2103,17 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t xml:space="preserve">Klassifikasjon</t>
+          <t xml:space="preserve">IDS-fasetter</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t xml:space="preserve">Rolle</t>
+          <t xml:space="preserve">Kardinalitet</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t xml:space="preserve">rules[].mapping</t>
+          <t xml:space="preserve">cardinality</t>
         </is>
       </c>
       <c r="D100" t="inlineStr">
@@ -2131,51 +2121,36 @@
           <t xml:space="preserve">text</t>
         </is>
       </c>
-      <c r="E100" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
-        </is>
-      </c>
       <c r="F100" t="inlineStr">
         <is>
-          <t xml:space="preserve">system-classification, component-classification</t>
+          <t xml:space="preserve">required, optional, prohibited</t>
         </is>
       </c>
       <c r="G100" t="inlineStr">
         <is>
-          <t xml:space="preserve">component-classification</t>
+          <t xml:space="preserve">required</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t xml:space="preserve">Klassifikasjon</t>
+          <t xml:space="preserve">IDS-fasetter</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t xml:space="preserve">ID</t>
+          <t xml:space="preserve">Instruksjon</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t xml:space="preserve">rules[].id</t>
+          <t xml:space="preserve">instructions</t>
         </is>
       </c>
       <c r="D101" t="inlineStr">
         <is>
           <t xml:space="preserve">text</t>
-        </is>
-      </c>
-      <c r="E101" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
-        </is>
-      </c>
-      <c r="G101" t="inlineStr">
-        <is>
-          <t xml:space="preserve">component-classification</t>
         </is>
       </c>
     </row>
@@ -2187,12 +2162,12 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t xml:space="preserve">Navn</t>
+          <t xml:space="preserve">Rolle</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t xml:space="preserve">rules[].name</t>
+          <t xml:space="preserve">rules[].mapping</t>
         </is>
       </c>
       <c r="D102" t="inlineStr">
@@ -2205,9 +2180,14 @@
           <t xml:space="preserve">yes</t>
         </is>
       </c>
+      <c r="F102" t="inlineStr">
+        <is>
+          <t xml:space="preserve">system-classification, component-classification</t>
+        </is>
+      </c>
       <c r="G102" t="inlineStr">
         <is>
-          <t xml:space="preserve">Komponentklasse</t>
+          <t xml:space="preserve">component-classification</t>
         </is>
       </c>
     </row>
@@ -2219,17 +2199,27 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t xml:space="preserve">Beskrivelse</t>
+          <t xml:space="preserve">ID</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t xml:space="preserve">rules[].description</t>
+          <t xml:space="preserve">rules[].id</t>
         </is>
       </c>
       <c r="D103" t="inlineStr">
         <is>
           <t xml:space="preserve">text</t>
+        </is>
+      </c>
+      <c r="E103" t="inlineStr">
+        <is>
+          <t xml:space="preserve">yes</t>
+        </is>
+      </c>
+      <c r="G103" t="inlineStr">
+        <is>
+          <t xml:space="preserve">component-classification</t>
         </is>
       </c>
     </row>
@@ -2241,12 +2231,12 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t xml:space="preserve">Referanse</t>
+          <t xml:space="preserve">Navn</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t xml:space="preserve">rules[].reference</t>
+          <t xml:space="preserve">rules[].name</t>
         </is>
       </c>
       <c r="D104" t="inlineStr">
@@ -2254,9 +2244,14 @@
           <t xml:space="preserve">text</t>
         </is>
       </c>
+      <c r="E104" t="inlineStr">
+        <is>
+          <t xml:space="preserve">yes</t>
+        </is>
+      </c>
       <c r="G104" t="inlineStr">
         <is>
-          <t xml:space="preserve">BEP §6.12</t>
+          <t xml:space="preserve">Komponentklasse</t>
         </is>
       </c>
     </row>
@@ -2268,32 +2263,17 @@
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t xml:space="preserve">Kodeliste</t>
+          <t xml:space="preserve">Beskrivelse</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t xml:space="preserve">rules[].check.list</t>
+          <t xml:space="preserve">rules[].description</t>
         </is>
       </c>
       <c r="D105" t="inlineStr">
         <is>
           <t xml:space="preserve">text</t>
-        </is>
-      </c>
-      <c r="E105" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
-        </is>
-      </c>
-      <c r="F105" t="inlineStr">
-        <is>
-          <t xml:space="preserve">ns3457-8, ns3451</t>
-        </is>
-      </c>
-      <c r="G105" t="inlineStr">
-        <is>
-          <t xml:space="preserve">ns3457-8</t>
         </is>
       </c>
     </row>
@@ -2305,12 +2285,12 @@
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t xml:space="preserve">Gjelder</t>
+          <t xml:space="preserve">Referanse</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t xml:space="preserve">rules[].check.target</t>
+          <t xml:space="preserve">rules[].reference</t>
         </is>
       </c>
       <c r="D106" t="inlineStr">
@@ -2318,14 +2298,9 @@
           <t xml:space="preserve">text</t>
         </is>
       </c>
-      <c r="F106" t="inlineStr">
-        <is>
-          <t xml:space="preserve">occurrence, type</t>
-        </is>
-      </c>
       <c r="G106" t="inlineStr">
         <is>
-          <t xml:space="preserve">type</t>
+          <t xml:space="preserve">BEP §6.12</t>
         </is>
       </c>
     </row>
@@ -2337,22 +2312,32 @@
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t xml:space="preserve">Nivå</t>
+          <t xml:space="preserve">Kodeliste</t>
         </is>
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t xml:space="preserve">rules[].check.minLevel</t>
+          <t xml:space="preserve">rules[].check.list</t>
         </is>
       </c>
       <c r="D107" t="inlineStr">
         <is>
-          <t xml:space="preserve">number</t>
+          <t xml:space="preserve">text</t>
+        </is>
+      </c>
+      <c r="E107" t="inlineStr">
+        <is>
+          <t xml:space="preserve">yes</t>
+        </is>
+      </c>
+      <c r="F107" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ns3457-8, ns3451</t>
         </is>
       </c>
       <c r="G107" t="inlineStr">
         <is>
-          <t xml:space="preserve">3</t>
+          <t xml:space="preserve">ns3457-8</t>
         </is>
       </c>
     </row>
@@ -2364,32 +2349,27 @@
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t xml:space="preserve">Kildetype</t>
+          <t xml:space="preserve">Gjelder</t>
         </is>
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t xml:space="preserve">rules[].check.source</t>
+          <t xml:space="preserve">rules[].check.target</t>
         </is>
       </c>
       <c r="D108" t="inlineStr">
         <is>
-          <t xml:space="preserve">source kind</t>
-        </is>
-      </c>
-      <c r="E108" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
+          <t xml:space="preserve">text</t>
         </is>
       </c>
       <c r="F108" t="inlineStr">
         <is>
-          <t xml:space="preserve">attribute, property, classification, material, progressCode</t>
+          <t xml:space="preserve">occurrence, type</t>
         </is>
       </c>
       <c r="G108" t="inlineStr">
         <is>
-          <t xml:space="preserve">attribute</t>
+          <t xml:space="preserve">type</t>
         </is>
       </c>
     </row>
@@ -2401,22 +2381,22 @@
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t xml:space="preserve">Attributt</t>
+          <t xml:space="preserve">Nivå</t>
         </is>
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t xml:space="preserve">rules[].check.source.attribute</t>
+          <t xml:space="preserve">rules[].check.minLevel</t>
         </is>
       </c>
       <c r="D109" t="inlineStr">
         <is>
-          <t xml:space="preserve">text</t>
+          <t xml:space="preserve">number</t>
         </is>
       </c>
       <c r="G109" t="inlineStr">
         <is>
-          <t xml:space="preserve">Name</t>
+          <t xml:space="preserve">3</t>
         </is>
       </c>
     </row>
@@ -2428,22 +2408,32 @@
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t xml:space="preserve">Egenskapssett</t>
+          <t xml:space="preserve">Kildetype</t>
         </is>
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t xml:space="preserve">rules[].check.source.property.propertySet</t>
+          <t xml:space="preserve">rules[].check.source</t>
         </is>
       </c>
       <c r="D110" t="inlineStr">
         <is>
-          <t xml:space="preserve">text</t>
+          <t xml:space="preserve">source kind</t>
+        </is>
+      </c>
+      <c r="E110" t="inlineStr">
+        <is>
+          <t xml:space="preserve">yes</t>
+        </is>
+      </c>
+      <c r="F110" t="inlineStr">
+        <is>
+          <t xml:space="preserve">attribute, property, classification, material, progressCode</t>
         </is>
       </c>
       <c r="G110" t="inlineStr">
         <is>
-          <t xml:space="preserve">EKS_Project</t>
+          <t xml:space="preserve">attribute</t>
         </is>
       </c>
     </row>
@@ -2455,12 +2445,12 @@
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t xml:space="preserve">Egenskapsnavn</t>
+          <t xml:space="preserve">Attributt</t>
         </is>
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t xml:space="preserve">rules[].check.source.property.name</t>
+          <t xml:space="preserve">rules[].check.source.attribute</t>
         </is>
       </c>
       <c r="D111" t="inlineStr">
@@ -2470,7 +2460,7 @@
       </c>
       <c r="G111" t="inlineStr">
         <is>
-          <t xml:space="preserve">MMI</t>
+          <t xml:space="preserve">Name</t>
         </is>
       </c>
     </row>
@@ -2482,12 +2472,12 @@
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t xml:space="preserve">System</t>
+          <t xml:space="preserve">Egenskapssett</t>
         </is>
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t xml:space="preserve">rules[].check.source.classification.system</t>
+          <t xml:space="preserve">rules[].check.source.property.propertySet</t>
         </is>
       </c>
       <c r="D112" t="inlineStr">
@@ -2497,7 +2487,7 @@
       </c>
       <c r="G112" t="inlineStr">
         <is>
-          <t xml:space="preserve">NS 3451</t>
+          <t xml:space="preserve">EKS_Project</t>
         </is>
       </c>
     </row>
@@ -2509,12 +2499,12 @@
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t xml:space="preserve">Uttrekk (regex)</t>
+          <t xml:space="preserve">Egenskapsnavn</t>
         </is>
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t xml:space="preserve">rules[].check.extract</t>
+          <t xml:space="preserve">rules[].check.source.property.name</t>
         </is>
       </c>
       <c r="D113" t="inlineStr">
@@ -2522,14 +2512,9 @@
           <t xml:space="preserve">text</t>
         </is>
       </c>
-      <c r="E113" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
-        </is>
-      </c>
       <c r="G113" t="inlineStr">
         <is>
-          <t xml:space="preserve">^([A-Z]{2,3})-\d{2}$</t>
+          <t xml:space="preserve">MMI</t>
         </is>
       </c>
     </row>
@@ -2541,32 +2526,22 @@
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t xml:space="preserve">Aktiv</t>
+          <t xml:space="preserve">System</t>
         </is>
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t xml:space="preserve">rules[].enabled</t>
+          <t xml:space="preserve">rules[].check.source.classification.system</t>
         </is>
       </c>
       <c r="D114" t="inlineStr">
         <is>
-          <t xml:space="preserve">TRUE / FALSE</t>
-        </is>
-      </c>
-      <c r="E114" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
-        </is>
-      </c>
-      <c r="F114" t="inlineStr">
-        <is>
-          <t xml:space="preserve">TRUE, FALSE</t>
+          <t xml:space="preserve">text</t>
         </is>
       </c>
       <c r="G114" t="inlineStr">
         <is>
-          <t xml:space="preserve">TRUE</t>
+          <t xml:space="preserve">NS 3451</t>
         </is>
       </c>
     </row>
@@ -2578,22 +2553,27 @@
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t xml:space="preserve">Utvalg</t>
+          <t xml:space="preserve">Uttrekk (regex)</t>
         </is>
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t xml:space="preserve">rules[].select</t>
+          <t xml:space="preserve">rules[].check.extract</t>
         </is>
       </c>
       <c r="D115" t="inlineStr">
         <is>
-          <t xml:space="preserve">JSON</t>
+          <t xml:space="preserve">text</t>
+        </is>
+      </c>
+      <c r="E115" t="inlineStr">
+        <is>
+          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="G115" t="inlineStr">
         <is>
-          <t xml:space="preserve">{"entity":{"group":"physicalElement"}}</t>
+          <t xml:space="preserve">^([A-Z]{2,3})-\d{2}$</t>
         </is>
       </c>
     </row>
@@ -2605,81 +2585,81 @@
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t xml:space="preserve">Instruksjon</t>
+          <t xml:space="preserve">Aktiv</t>
         </is>
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t xml:space="preserve">rules[].instructions</t>
+          <t xml:space="preserve">rules[].enabled</t>
         </is>
       </c>
       <c r="D116" t="inlineStr">
         <is>
-          <t xml:space="preserve">text</t>
+          <t xml:space="preserve">TRUE / FALSE</t>
+        </is>
+      </c>
+      <c r="E116" t="inlineStr">
+        <is>
+          <t xml:space="preserve">yes</t>
+        </is>
+      </c>
+      <c r="F116" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TRUE, FALSE</t>
+        </is>
+      </c>
+      <c r="G116" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TRUE</t>
         </is>
       </c>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t xml:space="preserve">MMI</t>
+          <t xml:space="preserve">Klassifikasjon</t>
         </is>
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t xml:space="preserve">ID</t>
+          <t xml:space="preserve">Utvalg</t>
         </is>
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t xml:space="preserve">rules[].id</t>
+          <t xml:space="preserve">rules[].select</t>
         </is>
       </c>
       <c r="D117" t="inlineStr">
         <is>
-          <t xml:space="preserve">text</t>
-        </is>
-      </c>
-      <c r="E117" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
+          <t xml:space="preserve">JSON</t>
         </is>
       </c>
       <c r="G117" t="inlineStr">
         <is>
-          <t xml:space="preserve">progress-code</t>
+          <t xml:space="preserve">{"entity":{"group":"physicalElement"}}</t>
         </is>
       </c>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t xml:space="preserve">MMI</t>
+          <t xml:space="preserve">Klassifikasjon</t>
         </is>
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t xml:space="preserve">Navn</t>
+          <t xml:space="preserve">Instruksjon</t>
         </is>
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t xml:space="preserve">rules[].name</t>
+          <t xml:space="preserve">rules[].instructions</t>
         </is>
       </c>
       <c r="D118" t="inlineStr">
         <is>
           <t xml:space="preserve">text</t>
-        </is>
-      </c>
-      <c r="E118" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
-        </is>
-      </c>
-      <c r="G118" t="inlineStr">
-        <is>
-          <t xml:space="preserve">MMI</t>
         </is>
       </c>
     </row>
@@ -2691,17 +2671,27 @@
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t xml:space="preserve">Beskrivelse</t>
+          <t xml:space="preserve">ID</t>
         </is>
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t xml:space="preserve">rules[].description</t>
+          <t xml:space="preserve">rules[].id</t>
         </is>
       </c>
       <c r="D119" t="inlineStr">
         <is>
           <t xml:space="preserve">text</t>
+        </is>
+      </c>
+      <c r="E119" t="inlineStr">
+        <is>
+          <t xml:space="preserve">yes</t>
+        </is>
+      </c>
+      <c r="G119" t="inlineStr">
+        <is>
+          <t xml:space="preserve">progress-code</t>
         </is>
       </c>
     </row>
@@ -2713,12 +2703,12 @@
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t xml:space="preserve">Referanse</t>
+          <t xml:space="preserve">Navn</t>
         </is>
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t xml:space="preserve">rules[].reference</t>
+          <t xml:space="preserve">rules[].name</t>
         </is>
       </c>
       <c r="D120" t="inlineStr">
@@ -2726,9 +2716,14 @@
           <t xml:space="preserve">text</t>
         </is>
       </c>
+      <c r="E120" t="inlineStr">
+        <is>
+          <t xml:space="preserve">yes</t>
+        </is>
+      </c>
       <c r="G120" t="inlineStr">
         <is>
-          <t xml:space="preserve">BEP §6.12</t>
+          <t xml:space="preserve">MMI</t>
         </is>
       </c>
     </row>
@@ -2740,32 +2735,17 @@
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t xml:space="preserve">Kildetype</t>
+          <t xml:space="preserve">Beskrivelse</t>
         </is>
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t xml:space="preserve">rules[].check.source</t>
+          <t xml:space="preserve">rules[].description</t>
         </is>
       </c>
       <c r="D121" t="inlineStr">
         <is>
-          <t xml:space="preserve">source kind</t>
-        </is>
-      </c>
-      <c r="E121" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
-        </is>
-      </c>
-      <c r="F121" t="inlineStr">
-        <is>
-          <t xml:space="preserve">attribute, property, classification, material, progressCode</t>
-        </is>
-      </c>
-      <c r="G121" t="inlineStr">
-        <is>
-          <t xml:space="preserve">property</t>
+          <t xml:space="preserve">text</t>
         </is>
       </c>
     </row>
@@ -2777,12 +2757,12 @@
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t xml:space="preserve">Attributt</t>
+          <t xml:space="preserve">Referanse</t>
         </is>
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t xml:space="preserve">rules[].check.source.attribute</t>
+          <t xml:space="preserve">rules[].reference</t>
         </is>
       </c>
       <c r="D122" t="inlineStr">
@@ -2792,7 +2772,7 @@
       </c>
       <c r="G122" t="inlineStr">
         <is>
-          <t xml:space="preserve">Name</t>
+          <t xml:space="preserve">BEP §6.12</t>
         </is>
       </c>
     </row>
@@ -2804,22 +2784,32 @@
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t xml:space="preserve">Egenskapssett</t>
+          <t xml:space="preserve">Kildetype</t>
         </is>
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t xml:space="preserve">rules[].check.source.property.propertySet</t>
+          <t xml:space="preserve">rules[].check.source</t>
         </is>
       </c>
       <c r="D123" t="inlineStr">
         <is>
-          <t xml:space="preserve">text</t>
+          <t xml:space="preserve">source kind</t>
+        </is>
+      </c>
+      <c r="E123" t="inlineStr">
+        <is>
+          <t xml:space="preserve">yes</t>
+        </is>
+      </c>
+      <c r="F123" t="inlineStr">
+        <is>
+          <t xml:space="preserve">attribute, property, classification, material, progressCode</t>
         </is>
       </c>
       <c r="G123" t="inlineStr">
         <is>
-          <t xml:space="preserve">EKS_Project</t>
+          <t xml:space="preserve">property</t>
         </is>
       </c>
     </row>
@@ -2831,12 +2821,12 @@
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t xml:space="preserve">Egenskapsnavn</t>
+          <t xml:space="preserve">Attributt</t>
         </is>
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t xml:space="preserve">rules[].check.source.property.name</t>
+          <t xml:space="preserve">rules[].check.source.attribute</t>
         </is>
       </c>
       <c r="D124" t="inlineStr">
@@ -2846,7 +2836,7 @@
       </c>
       <c r="G124" t="inlineStr">
         <is>
-          <t xml:space="preserve">MMI</t>
+          <t xml:space="preserve">Name</t>
         </is>
       </c>
     </row>
@@ -2858,12 +2848,12 @@
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t xml:space="preserve">System</t>
+          <t xml:space="preserve">Egenskapssett</t>
         </is>
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t xml:space="preserve">rules[].check.source.classification.system</t>
+          <t xml:space="preserve">rules[].check.source.property.propertySet</t>
         </is>
       </c>
       <c r="D125" t="inlineStr">
@@ -2873,7 +2863,7 @@
       </c>
       <c r="G125" t="inlineStr">
         <is>
-          <t xml:space="preserve">NS 3451</t>
+          <t xml:space="preserve">EKS_Project</t>
         </is>
       </c>
     </row>
@@ -2885,12 +2875,12 @@
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t xml:space="preserve">Uttrekk (regex)</t>
+          <t xml:space="preserve">Egenskapsnavn</t>
         </is>
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t xml:space="preserve">rules[].check.extract</t>
+          <t xml:space="preserve">rules[].check.source.property.name</t>
         </is>
       </c>
       <c r="D126" t="inlineStr">
@@ -2898,14 +2888,9 @@
           <t xml:space="preserve">text</t>
         </is>
       </c>
-      <c r="E126" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
-        </is>
-      </c>
       <c r="G126" t="inlineStr">
         <is>
-          <t xml:space="preserve">^(\d{3})$</t>
+          <t xml:space="preserve">MMI</t>
         </is>
       </c>
     </row>
@@ -2917,32 +2902,22 @@
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t xml:space="preserve">Aktiv</t>
+          <t xml:space="preserve">System</t>
         </is>
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t xml:space="preserve">rules[].enabled</t>
+          <t xml:space="preserve">rules[].check.source.classification.system</t>
         </is>
       </c>
       <c r="D127" t="inlineStr">
         <is>
-          <t xml:space="preserve">TRUE / FALSE</t>
-        </is>
-      </c>
-      <c r="E127" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
-        </is>
-      </c>
-      <c r="F127" t="inlineStr">
-        <is>
-          <t xml:space="preserve">TRUE, FALSE</t>
+          <t xml:space="preserve">text</t>
         </is>
       </c>
       <c r="G127" t="inlineStr">
         <is>
-          <t xml:space="preserve">TRUE</t>
+          <t xml:space="preserve">NS 3451</t>
         </is>
       </c>
     </row>
@@ -2954,22 +2929,27 @@
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t xml:space="preserve">Utvalg</t>
+          <t xml:space="preserve">Uttrekk (regex)</t>
         </is>
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t xml:space="preserve">rules[].select</t>
+          <t xml:space="preserve">rules[].check.extract</t>
         </is>
       </c>
       <c r="D128" t="inlineStr">
         <is>
-          <t xml:space="preserve">JSON</t>
+          <t xml:space="preserve">text</t>
+        </is>
+      </c>
+      <c r="E128" t="inlineStr">
+        <is>
+          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="G128" t="inlineStr">
         <is>
-          <t xml:space="preserve">{"entity":{"group":"physicalElement"}}</t>
+          <t xml:space="preserve">^(\d{3})$</t>
         </is>
       </c>
     </row>
@@ -2981,81 +2961,81 @@
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t xml:space="preserve">Instruksjon</t>
+          <t xml:space="preserve">Aktiv</t>
         </is>
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t xml:space="preserve">rules[].instructions</t>
+          <t xml:space="preserve">rules[].enabled</t>
         </is>
       </c>
       <c r="D129" t="inlineStr">
         <is>
-          <t xml:space="preserve">text</t>
+          <t xml:space="preserve">TRUE / FALSE</t>
+        </is>
+      </c>
+      <c r="E129" t="inlineStr">
+        <is>
+          <t xml:space="preserve">yes</t>
+        </is>
+      </c>
+      <c r="F129" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TRUE, FALSE</t>
+        </is>
+      </c>
+      <c r="G129" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TRUE</t>
         </is>
       </c>
     </row>
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t xml:space="preserve">MMI-koder</t>
+          <t xml:space="preserve">MMI</t>
         </is>
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t xml:space="preserve">Kode</t>
+          <t xml:space="preserve">Utvalg</t>
         </is>
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t xml:space="preserve">rules[].check.codes[].code</t>
+          <t xml:space="preserve">rules[].select</t>
         </is>
       </c>
       <c r="D130" t="inlineStr">
         <is>
-          <t xml:space="preserve">text</t>
-        </is>
-      </c>
-      <c r="E130" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
+          <t xml:space="preserve">JSON</t>
         </is>
       </c>
       <c r="G130" t="inlineStr">
         <is>
-          <t xml:space="preserve">300</t>
+          <t xml:space="preserve">{"entity":{"group":"physicalElement"}}</t>
         </is>
       </c>
     </row>
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t xml:space="preserve">MMI-koder</t>
+          <t xml:space="preserve">MMI</t>
         </is>
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t xml:space="preserve">Navn</t>
+          <t xml:space="preserve">Instruksjon</t>
         </is>
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t xml:space="preserve">rules[].check.codes[].name</t>
+          <t xml:space="preserve">rules[].instructions</t>
         </is>
       </c>
       <c r="D131" t="inlineStr">
         <is>
           <t xml:space="preserve">text</t>
-        </is>
-      </c>
-      <c r="E131" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
-        </is>
-      </c>
-      <c r="G131" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Detaljprosjektert</t>
         </is>
       </c>
     </row>
@@ -3067,12 +3047,12 @@
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t xml:space="preserve">Fase</t>
+          <t xml:space="preserve">Kode</t>
         </is>
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t xml:space="preserve">rules[].check.codes[].phase</t>
+          <t xml:space="preserve">rules[].check.codes[].code</t>
         </is>
       </c>
       <c r="D132" t="inlineStr">
@@ -3080,26 +3060,31 @@
           <t xml:space="preserve">text</t>
         </is>
       </c>
+      <c r="E132" t="inlineStr">
+        <is>
+          <t xml:space="preserve">yes</t>
+        </is>
+      </c>
       <c r="G132" t="inlineStr">
         <is>
-          <t xml:space="preserve">NY</t>
+          <t xml:space="preserve">300</t>
         </is>
       </c>
     </row>
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t xml:space="preserve">Kopiobjekt</t>
+          <t xml:space="preserve">MMI-koder</t>
         </is>
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t xml:space="preserve">ID</t>
+          <t xml:space="preserve">Navn</t>
         </is>
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t xml:space="preserve">rules[].id</t>
+          <t xml:space="preserve">rules[].check.codes[].name</t>
         </is>
       </c>
       <c r="D133" t="inlineStr">
@@ -3114,24 +3099,24 @@
       </c>
       <c r="G133" t="inlineStr">
         <is>
-          <t xml:space="preserve">copy-object</t>
+          <t xml:space="preserve">Detaljprosjektert</t>
         </is>
       </c>
     </row>
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t xml:space="preserve">Kopiobjekt</t>
+          <t xml:space="preserve">MMI-koder</t>
         </is>
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t xml:space="preserve">Navn</t>
+          <t xml:space="preserve">Fase</t>
         </is>
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t xml:space="preserve">rules[].name</t>
+          <t xml:space="preserve">rules[].check.codes[].phase</t>
         </is>
       </c>
       <c r="D134" t="inlineStr">
@@ -3139,14 +3124,9 @@
           <t xml:space="preserve">text</t>
         </is>
       </c>
-      <c r="E134" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
-        </is>
-      </c>
       <c r="G134" t="inlineStr">
         <is>
-          <t xml:space="preserve">Kopiobjekt</t>
+          <t xml:space="preserve">NY</t>
         </is>
       </c>
     </row>
@@ -3158,17 +3138,27 @@
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t xml:space="preserve">Beskrivelse</t>
+          <t xml:space="preserve">ID</t>
         </is>
       </c>
       <c r="C135" t="inlineStr">
         <is>
-          <t xml:space="preserve">rules[].description</t>
+          <t xml:space="preserve">rules[].id</t>
         </is>
       </c>
       <c r="D135" t="inlineStr">
         <is>
           <t xml:space="preserve">text</t>
+        </is>
+      </c>
+      <c r="E135" t="inlineStr">
+        <is>
+          <t xml:space="preserve">yes</t>
+        </is>
+      </c>
+      <c r="G135" t="inlineStr">
+        <is>
+          <t xml:space="preserve">copy-object</t>
         </is>
       </c>
     </row>
@@ -3180,12 +3170,12 @@
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t xml:space="preserve">Referanse</t>
+          <t xml:space="preserve">Navn</t>
         </is>
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t xml:space="preserve">rules[].reference</t>
+          <t xml:space="preserve">rules[].name</t>
         </is>
       </c>
       <c r="D136" t="inlineStr">
@@ -3193,9 +3183,14 @@
           <t xml:space="preserve">text</t>
         </is>
       </c>
+      <c r="E136" t="inlineStr">
+        <is>
+          <t xml:space="preserve">yes</t>
+        </is>
+      </c>
       <c r="G136" t="inlineStr">
         <is>
-          <t xml:space="preserve">BEP §6.12</t>
+          <t xml:space="preserve">Kopiobjekt</t>
         </is>
       </c>
     </row>
@@ -3207,32 +3202,17 @@
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t xml:space="preserve">Kildetype</t>
+          <t xml:space="preserve">Beskrivelse</t>
         </is>
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t xml:space="preserve">rules[].check.source</t>
+          <t xml:space="preserve">rules[].description</t>
         </is>
       </c>
       <c r="D137" t="inlineStr">
         <is>
-          <t xml:space="preserve">source kind</t>
-        </is>
-      </c>
-      <c r="E137" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
-        </is>
-      </c>
-      <c r="F137" t="inlineStr">
-        <is>
-          <t xml:space="preserve">attribute, property, classification, material, progressCode</t>
-        </is>
-      </c>
-      <c r="G137" t="inlineStr">
-        <is>
-          <t xml:space="preserve">property</t>
+          <t xml:space="preserve">text</t>
         </is>
       </c>
     </row>
@@ -3244,12 +3224,12 @@
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t xml:space="preserve">Attributt</t>
+          <t xml:space="preserve">Referanse</t>
         </is>
       </c>
       <c r="C138" t="inlineStr">
         <is>
-          <t xml:space="preserve">rules[].check.source.attribute</t>
+          <t xml:space="preserve">rules[].reference</t>
         </is>
       </c>
       <c r="D138" t="inlineStr">
@@ -3259,7 +3239,7 @@
       </c>
       <c r="G138" t="inlineStr">
         <is>
-          <t xml:space="preserve">Name</t>
+          <t xml:space="preserve">BEP §6.12</t>
         </is>
       </c>
     </row>
@@ -3271,22 +3251,32 @@
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t xml:space="preserve">Egenskapssett</t>
+          <t xml:space="preserve">Kildetype</t>
         </is>
       </c>
       <c r="C139" t="inlineStr">
         <is>
-          <t xml:space="preserve">rules[].check.source.property.propertySet</t>
+          <t xml:space="preserve">rules[].check.source</t>
         </is>
       </c>
       <c r="D139" t="inlineStr">
         <is>
-          <t xml:space="preserve">text</t>
+          <t xml:space="preserve">source kind</t>
+        </is>
+      </c>
+      <c r="E139" t="inlineStr">
+        <is>
+          <t xml:space="preserve">yes</t>
+        </is>
+      </c>
+      <c r="F139" t="inlineStr">
+        <is>
+          <t xml:space="preserve">attribute, property, classification, material, progressCode</t>
         </is>
       </c>
       <c r="G139" t="inlineStr">
         <is>
-          <t xml:space="preserve">EKS_Project</t>
+          <t xml:space="preserve">property</t>
         </is>
       </c>
     </row>
@@ -3298,12 +3288,12 @@
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t xml:space="preserve">Egenskapsnavn</t>
+          <t xml:space="preserve">Attributt</t>
         </is>
       </c>
       <c r="C140" t="inlineStr">
         <is>
-          <t xml:space="preserve">rules[].check.source.property.name</t>
+          <t xml:space="preserve">rules[].check.source.attribute</t>
         </is>
       </c>
       <c r="D140" t="inlineStr">
@@ -3313,7 +3303,7 @@
       </c>
       <c r="G140" t="inlineStr">
         <is>
-          <t xml:space="preserve">MMI</t>
+          <t xml:space="preserve">Name</t>
         </is>
       </c>
     </row>
@@ -3325,12 +3315,12 @@
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t xml:space="preserve">System</t>
+          <t xml:space="preserve">Egenskapssett</t>
         </is>
       </c>
       <c r="C141" t="inlineStr">
         <is>
-          <t xml:space="preserve">rules[].check.source.classification.system</t>
+          <t xml:space="preserve">rules[].check.source.property.propertySet</t>
         </is>
       </c>
       <c r="D141" t="inlineStr">
@@ -3340,7 +3330,7 @@
       </c>
       <c r="G141" t="inlineStr">
         <is>
-          <t xml:space="preserve">NS 3451</t>
+          <t xml:space="preserve">EKS_Project</t>
         </is>
       </c>
     </row>
@@ -3352,22 +3342,22 @@
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t xml:space="preserve">Kopiverdier</t>
+          <t xml:space="preserve">Egenskapsnavn</t>
         </is>
       </c>
       <c r="C142" t="inlineStr">
         <is>
-          <t xml:space="preserve">rules[].check.copy</t>
+          <t xml:space="preserve">rules[].check.source.property.name</t>
         </is>
       </c>
       <c r="D142" t="inlineStr">
         <is>
-          <t xml:space="preserve">list, blank = none</t>
+          <t xml:space="preserve">text</t>
         </is>
       </c>
       <c r="G142" t="inlineStr">
         <is>
-          <t xml:space="preserve">true, ja, kopi</t>
+          <t xml:space="preserve">MMI</t>
         </is>
       </c>
     </row>
@@ -3379,22 +3369,22 @@
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t xml:space="preserve">Egne verdier</t>
+          <t xml:space="preserve">System</t>
         </is>
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t xml:space="preserve">rules[].check.own</t>
+          <t xml:space="preserve">rules[].check.source.classification.system</t>
         </is>
       </c>
       <c r="D143" t="inlineStr">
         <is>
-          <t xml:space="preserve">list, blank = none</t>
+          <t xml:space="preserve">text</t>
         </is>
       </c>
       <c r="G143" t="inlineStr">
         <is>
-          <t xml:space="preserve">false, nei</t>
+          <t xml:space="preserve">NS 3451</t>
         </is>
       </c>
     </row>
@@ -3406,32 +3396,22 @@
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t xml:space="preserve">Aktiv</t>
+          <t xml:space="preserve">Kopiverdier</t>
         </is>
       </c>
       <c r="C144" t="inlineStr">
         <is>
-          <t xml:space="preserve">rules[].enabled</t>
+          <t xml:space="preserve">rules[].check.copy</t>
         </is>
       </c>
       <c r="D144" t="inlineStr">
         <is>
-          <t xml:space="preserve">TRUE / FALSE</t>
-        </is>
-      </c>
-      <c r="E144" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
-        </is>
-      </c>
-      <c r="F144" t="inlineStr">
-        <is>
-          <t xml:space="preserve">TRUE, FALSE</t>
+          <t xml:space="preserve">list, blank = none</t>
         </is>
       </c>
       <c r="G144" t="inlineStr">
         <is>
-          <t xml:space="preserve">TRUE</t>
+          <t xml:space="preserve">true, ja, kopi</t>
         </is>
       </c>
     </row>
@@ -3443,22 +3423,22 @@
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t xml:space="preserve">Utvalg</t>
+          <t xml:space="preserve">Egne verdier</t>
         </is>
       </c>
       <c r="C145" t="inlineStr">
         <is>
-          <t xml:space="preserve">rules[].select</t>
+          <t xml:space="preserve">rules[].check.own</t>
         </is>
       </c>
       <c r="D145" t="inlineStr">
         <is>
-          <t xml:space="preserve">JSON</t>
+          <t xml:space="preserve">list, blank = none</t>
         </is>
       </c>
       <c r="G145" t="inlineStr">
         <is>
-          <t xml:space="preserve">{"entity":{"group":"physicalElement"}}</t>
+          <t xml:space="preserve">false, nei</t>
         </is>
       </c>
     </row>
@@ -3470,81 +3450,81 @@
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t xml:space="preserve">Instruksjon</t>
+          <t xml:space="preserve">Aktiv</t>
         </is>
       </c>
       <c r="C146" t="inlineStr">
         <is>
-          <t xml:space="preserve">rules[].instructions</t>
+          <t xml:space="preserve">rules[].enabled</t>
         </is>
       </c>
       <c r="D146" t="inlineStr">
         <is>
-          <t xml:space="preserve">text</t>
+          <t xml:space="preserve">TRUE / FALSE</t>
+        </is>
+      </c>
+      <c r="E146" t="inlineStr">
+        <is>
+          <t xml:space="preserve">yes</t>
+        </is>
+      </c>
+      <c r="F146" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TRUE, FALSE</t>
+        </is>
+      </c>
+      <c r="G146" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TRUE</t>
         </is>
       </c>
     </row>
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t xml:space="preserve">Etasjeoppsett</t>
+          <t xml:space="preserve">Kopiobjekt</t>
         </is>
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t xml:space="preserve">Fagkode</t>
+          <t xml:space="preserve">Utvalg</t>
         </is>
       </c>
       <c r="C147" t="inlineStr">
         <is>
-          <t xml:space="preserve">discipline</t>
+          <t xml:space="preserve">rules[].select</t>
         </is>
       </c>
       <c r="D147" t="inlineStr">
         <is>
-          <t xml:space="preserve">text</t>
+          <t xml:space="preserve">JSON</t>
         </is>
       </c>
       <c r="G147" t="inlineStr">
         <is>
-          <t xml:space="preserve">RIB</t>
+          <t xml:space="preserve">{"entity":{"group":"physicalElement"}}</t>
         </is>
       </c>
     </row>
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t xml:space="preserve">Etasjeoppsett</t>
+          <t xml:space="preserve">Kopiobjekt</t>
         </is>
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t xml:space="preserve">Referanseplan</t>
+          <t xml:space="preserve">Instruksjon</t>
         </is>
       </c>
       <c r="C148" t="inlineStr">
         <is>
-          <t xml:space="preserve">plane</t>
+          <t xml:space="preserve">rules[].instructions</t>
         </is>
       </c>
       <c r="D148" t="inlineStr">
         <is>
           <t xml:space="preserve">text</t>
-        </is>
-      </c>
-      <c r="E148" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
-        </is>
-      </c>
-      <c r="F148" t="inlineStr">
-        <is>
-          <t xml:space="preserve">OKFG, OKBD</t>
-        </is>
-      </c>
-      <c r="G148" t="inlineStr">
-        <is>
-          <t xml:space="preserve">OKFG</t>
         </is>
       </c>
     </row>
@@ -3556,22 +3536,22 @@
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t xml:space="preserve">Toleranse over (mm)</t>
+          <t xml:space="preserve">Fagkode</t>
         </is>
       </c>
       <c r="C149" t="inlineStr">
         <is>
-          <t xml:space="preserve">tolerance.aboveMm</t>
+          <t xml:space="preserve">discipline</t>
         </is>
       </c>
       <c r="D149" t="inlineStr">
         <is>
-          <t xml:space="preserve">mm, blank = no limit</t>
+          <t xml:space="preserve">text</t>
         </is>
       </c>
       <c r="G149" t="inlineStr">
         <is>
-          <t xml:space="preserve">5</t>
+          <t xml:space="preserve">RIB</t>
         </is>
       </c>
     </row>
@@ -3583,22 +3563,32 @@
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t xml:space="preserve">Toleranse under (mm)</t>
+          <t xml:space="preserve">Referanseplan</t>
         </is>
       </c>
       <c r="C150" t="inlineStr">
         <is>
-          <t xml:space="preserve">tolerance.belowMm</t>
+          <t xml:space="preserve">plane</t>
         </is>
       </c>
       <c r="D150" t="inlineStr">
         <is>
-          <t xml:space="preserve">mm, blank = no limit</t>
+          <t xml:space="preserve">text</t>
+        </is>
+      </c>
+      <c r="E150" t="inlineStr">
+        <is>
+          <t xml:space="preserve">yes</t>
+        </is>
+      </c>
+      <c r="F150" t="inlineStr">
+        <is>
+          <t xml:space="preserve">OKFG, OKBD</t>
         </is>
       </c>
       <c r="G150" t="inlineStr">
         <is>
-          <t xml:space="preserve">5</t>
+          <t xml:space="preserve">OKFG</t>
         </is>
       </c>
     </row>
@@ -3610,12 +3600,12 @@
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t xml:space="preserve">Navnevindu (mm)</t>
+          <t xml:space="preserve">Toleranse over (mm)</t>
         </is>
       </c>
       <c r="C151" t="inlineStr">
         <is>
-          <t xml:space="preserve">nameWindowMm</t>
+          <t xml:space="preserve">tolerance.aboveMm</t>
         </is>
       </c>
       <c r="D151" t="inlineStr">
@@ -3625,7 +3615,7 @@
       </c>
       <c r="G151" t="inlineStr">
         <is>
-          <t xml:space="preserve">1000</t>
+          <t xml:space="preserve">5</t>
         </is>
       </c>
     </row>
@@ -3637,22 +3627,22 @@
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t xml:space="preserve">Nærvindu (mm)</t>
+          <t xml:space="preserve">Toleranse under (mm)</t>
         </is>
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t xml:space="preserve">nearMm</t>
+          <t xml:space="preserve">tolerance.belowMm</t>
         </is>
       </c>
       <c r="D152" t="inlineStr">
         <is>
-          <t xml:space="preserve">number</t>
+          <t xml:space="preserve">mm, blank = no limit</t>
         </is>
       </c>
       <c r="G152" t="inlineStr">
         <is>
-          <t xml:space="preserve">200</t>
+          <t xml:space="preserve">5</t>
         </is>
       </c>
     </row>
@@ -3664,27 +3654,22 @@
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t xml:space="preserve">Alle navn må stemme</t>
+          <t xml:space="preserve">Navnevindu (mm)</t>
         </is>
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t xml:space="preserve">requireAllNames</t>
+          <t xml:space="preserve">nameWindowMm</t>
         </is>
       </c>
       <c r="D153" t="inlineStr">
         <is>
-          <t xml:space="preserve">TRUE / FALSE</t>
-        </is>
-      </c>
-      <c r="F153" t="inlineStr">
-        <is>
-          <t xml:space="preserve">TRUE, FALSE</t>
+          <t xml:space="preserve">mm, blank = no limit</t>
         </is>
       </c>
       <c r="G153" t="inlineStr">
         <is>
-          <t xml:space="preserve">TRUE</t>
+          <t xml:space="preserve">1000</t>
         </is>
       </c>
     </row>
@@ -3696,103 +3681,98 @@
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t xml:space="preserve">Referanse</t>
+          <t xml:space="preserve">Nærvindu (mm)</t>
         </is>
       </c>
       <c r="C154" t="inlineStr">
         <is>
-          <t xml:space="preserve">reference</t>
+          <t xml:space="preserve">nearMm</t>
         </is>
       </c>
       <c r="D154" t="inlineStr">
         <is>
-          <t xml:space="preserve">text</t>
+          <t xml:space="preserve">number</t>
         </is>
       </c>
       <c r="G154" t="inlineStr">
         <is>
-          <t xml:space="preserve">BEP §3.2</t>
+          <t xml:space="preserve">200</t>
         </is>
       </c>
     </row>
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
-          <t xml:space="preserve">Etasjer</t>
+          <t xml:space="preserve">Etasjeoppsett</t>
         </is>
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t xml:space="preserve">Navn</t>
+          <t xml:space="preserve">Alle navn må stemme</t>
         </is>
       </c>
       <c r="C155" t="inlineStr">
         <is>
-          <t xml:space="preserve">storeys.levels[].name</t>
+          <t xml:space="preserve">requireAllNames</t>
         </is>
       </c>
       <c r="D155" t="inlineStr">
         <is>
-          <t xml:space="preserve">text</t>
-        </is>
-      </c>
-      <c r="E155" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
+          <t xml:space="preserve">TRUE / FALSE</t>
+        </is>
+      </c>
+      <c r="F155" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TRUE, FALSE</t>
         </is>
       </c>
       <c r="G155" t="inlineStr">
         <is>
-          <t xml:space="preserve">Plan 01</t>
+          <t xml:space="preserve">TRUE</t>
         </is>
       </c>
     </row>
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
-          <t xml:space="preserve">Etasjer</t>
+          <t xml:space="preserve">Etasjeoppsett</t>
         </is>
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t xml:space="preserve">Kote (m)</t>
+          <t xml:space="preserve">Referanse</t>
         </is>
       </c>
       <c r="C156" t="inlineStr">
         <is>
-          <t xml:space="preserve">storeys.levels[].elevation</t>
+          <t xml:space="preserve">reference</t>
         </is>
       </c>
       <c r="D156" t="inlineStr">
         <is>
-          <t xml:space="preserve">number</t>
-        </is>
-      </c>
-      <c r="E156" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
+          <t xml:space="preserve">text</t>
         </is>
       </c>
       <c r="G156" t="inlineStr">
         <is>
-          <t xml:space="preserve">24.15</t>
+          <t xml:space="preserve">BEP §3.2</t>
         </is>
       </c>
     </row>
     <row r="157">
       <c r="A157" t="inlineStr">
         <is>
-          <t xml:space="preserve">Fag</t>
+          <t xml:space="preserve">Etasjer</t>
         </is>
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t xml:space="preserve">Fagkode</t>
+          <t xml:space="preserve">Navn</t>
         </is>
       </c>
       <c r="C157" t="inlineStr">
         <is>
-          <t xml:space="preserve">disciplines[].code</t>
+          <t xml:space="preserve">storeys.levels[].name</t>
         </is>
       </c>
       <c r="D157" t="inlineStr">
@@ -3807,29 +3787,29 @@
       </c>
       <c r="G157" t="inlineStr">
         <is>
-          <t xml:space="preserve">ARK</t>
+          <t xml:space="preserve">Plan 01</t>
         </is>
       </c>
     </row>
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t xml:space="preserve">Fag</t>
+          <t xml:space="preserve">Etasjer</t>
         </is>
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t xml:space="preserve">Rapport</t>
+          <t xml:space="preserve">Kote (m)</t>
         </is>
       </c>
       <c r="C158" t="inlineStr">
         <is>
-          <t xml:space="preserve">disciplines[].report</t>
+          <t xml:space="preserve">storeys.levels[].elevation</t>
         </is>
       </c>
       <c r="D158" t="inlineStr">
         <is>
-          <t xml:space="preserve">TRUE / FALSE</t>
+          <t xml:space="preserve">number</t>
         </is>
       </c>
       <c r="E158" t="inlineStr">
@@ -3837,31 +3817,26 @@
           <t xml:space="preserve">yes</t>
         </is>
       </c>
-      <c r="F158" t="inlineStr">
-        <is>
-          <t xml:space="preserve">TRUE, FALSE</t>
-        </is>
-      </c>
       <c r="G158" t="inlineStr">
         <is>
-          <t xml:space="preserve">TRUE</t>
+          <t xml:space="preserve">24.15</t>
         </is>
       </c>
     </row>
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t xml:space="preserve">Modeller</t>
+          <t xml:space="preserve">Fag</t>
         </is>
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t xml:space="preserve">Modell</t>
+          <t xml:space="preserve">Fagkode</t>
         </is>
       </c>
       <c r="C159" t="inlineStr">
         <is>
-          <t xml:space="preserve">models[].label</t>
+          <t xml:space="preserve">disciplines[].code</t>
         </is>
       </c>
       <c r="D159" t="inlineStr">
@@ -3876,29 +3851,29 @@
       </c>
       <c r="G159" t="inlineStr">
         <is>
-          <t xml:space="preserve">EKS_ARK</t>
+          <t xml:space="preserve">ARK</t>
         </is>
       </c>
     </row>
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t xml:space="preserve">Modeller</t>
+          <t xml:space="preserve">Fag</t>
         </is>
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t xml:space="preserve">Fagkode</t>
+          <t xml:space="preserve">Rapport</t>
         </is>
       </c>
       <c r="C160" t="inlineStr">
         <is>
-          <t xml:space="preserve">models[].discipline</t>
+          <t xml:space="preserve">disciplines[].report</t>
         </is>
       </c>
       <c r="D160" t="inlineStr">
         <is>
-          <t xml:space="preserve">text</t>
+          <t xml:space="preserve">TRUE / FALSE</t>
         </is>
       </c>
       <c r="E160" t="inlineStr">
@@ -3906,9 +3881,14 @@
           <t xml:space="preserve">yes</t>
         </is>
       </c>
+      <c r="F160" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TRUE, FALSE</t>
+        </is>
+      </c>
       <c r="G160" t="inlineStr">
         <is>
-          <t xml:space="preserve">ARK</t>
+          <t xml:space="preserve">TRUE</t>
         </is>
       </c>
     </row>
@@ -3920,12 +3900,12 @@
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t xml:space="preserve">Gruppe</t>
+          <t xml:space="preserve">Modell</t>
         </is>
       </c>
       <c r="C161" t="inlineStr">
         <is>
-          <t xml:space="preserve">models[].group</t>
+          <t xml:space="preserve">models[].label</t>
         </is>
       </c>
       <c r="D161" t="inlineStr">
@@ -3933,9 +3913,14 @@
           <t xml:space="preserve">text</t>
         </is>
       </c>
+      <c r="E161" t="inlineStr">
+        <is>
+          <t xml:space="preserve">yes</t>
+        </is>
+      </c>
       <c r="G161" t="inlineStr">
         <is>
-          <t xml:space="preserve">ARK</t>
+          <t xml:space="preserve">EKS_ARK</t>
         </is>
       </c>
     </row>
@@ -3947,22 +3932,27 @@
       </c>
       <c r="B162" t="inlineStr">
         <is>
-          <t xml:space="preserve">Eierverdier</t>
+          <t xml:space="preserve">Fagkode</t>
         </is>
       </c>
       <c r="C162" t="inlineStr">
         <is>
-          <t xml:space="preserve">models[].ownerNames</t>
+          <t xml:space="preserve">models[].discipline</t>
         </is>
       </c>
       <c r="D162" t="inlineStr">
         <is>
-          <t xml:space="preserve">list</t>
+          <t xml:space="preserve">text</t>
+        </is>
+      </c>
+      <c r="E162" t="inlineStr">
+        <is>
+          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="G162" t="inlineStr">
         <is>
-          <t xml:space="preserve">EKS_ARK, ARK</t>
+          <t xml:space="preserve">ARK</t>
         </is>
       </c>
     </row>
@@ -3974,86 +3964,76 @@
       </c>
       <c r="B163" t="inlineStr">
         <is>
-          <t xml:space="preserve">Gjelder ikke</t>
+          <t xml:space="preserve">Gruppe</t>
         </is>
       </c>
       <c r="C163" t="inlineStr">
         <is>
-          <t xml:space="preserve">models[].exempt</t>
+          <t xml:space="preserve">models[].group</t>
         </is>
       </c>
       <c r="D163" t="inlineStr">
         <is>
-          <t xml:space="preserve">list</t>
+          <t xml:space="preserve">text</t>
         </is>
       </c>
       <c r="G163" t="inlineStr">
         <is>
-          <t xml:space="preserve">system-classification, phase</t>
+          <t xml:space="preserve">ARK</t>
         </is>
       </c>
     </row>
     <row r="164">
       <c r="A164" t="inlineStr">
         <is>
-          <t xml:space="preserve">Standardkrav</t>
+          <t xml:space="preserve">Modeller</t>
         </is>
       </c>
       <c r="B164" t="inlineStr">
         <is>
-          <t xml:space="preserve">Krav</t>
+          <t xml:space="preserve">Eierverdier</t>
         </is>
       </c>
       <c r="C164" t="inlineStr">
         <is>
-          <t xml:space="preserve">projectLayer</t>
+          <t xml:space="preserve">models[].ownerNames</t>
         </is>
       </c>
       <c r="D164" t="inlineStr">
         <is>
-          <t xml:space="preserve">text</t>
-        </is>
-      </c>
-      <c r="E164" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
-        </is>
-      </c>
-      <c r="F164" t="inlineStr">
-        <is>
-          <t xml:space="preserve">ifc-schema, phase, material-product</t>
+          <t xml:space="preserve">list</t>
         </is>
       </c>
       <c r="G164" t="inlineStr">
         <is>
-          <t xml:space="preserve">ifc-schema</t>
+          <t xml:space="preserve">EKS_ARK, ARK</t>
         </is>
       </c>
     </row>
     <row r="165">
       <c r="A165" t="inlineStr">
         <is>
-          <t xml:space="preserve">Standardkrav</t>
+          <t xml:space="preserve">Modeller</t>
         </is>
       </c>
       <c r="B165" t="inlineStr">
         <is>
-          <t xml:space="preserve">Referanse</t>
+          <t xml:space="preserve">Gjelder ikke</t>
         </is>
       </c>
       <c r="C165" t="inlineStr">
         <is>
-          <t xml:space="preserve">reference</t>
+          <t xml:space="preserve">models[].exempt</t>
         </is>
       </c>
       <c r="D165" t="inlineStr">
         <is>
-          <t xml:space="preserve">text</t>
+          <t xml:space="preserve">list</t>
         </is>
       </c>
       <c r="G165" t="inlineStr">
         <is>
-          <t xml:space="preserve">BEP §3</t>
+          <t xml:space="preserve">system-classification, phase</t>
         </is>
       </c>
     </row>
@@ -4065,22 +4045,32 @@
       </c>
       <c r="B166" t="inlineStr">
         <is>
-          <t xml:space="preserve">Godtatte</t>
+          <t xml:space="preserve">Krav</t>
         </is>
       </c>
       <c r="C166" t="inlineStr">
         <is>
-          <t xml:space="preserve">accepted</t>
+          <t xml:space="preserve">projectLayer</t>
         </is>
       </c>
       <c r="D166" t="inlineStr">
         <is>
-          <t xml:space="preserve">list</t>
+          <t xml:space="preserve">text</t>
+        </is>
+      </c>
+      <c r="E166" t="inlineStr">
+        <is>
+          <t xml:space="preserve">yes</t>
+        </is>
+      </c>
+      <c r="F166" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ifc-schema, phase, material-product</t>
         </is>
       </c>
       <c r="G166" t="inlineStr">
         <is>
-          <t xml:space="preserve">IFC2X3, IFC4</t>
+          <t xml:space="preserve">ifc-schema</t>
         </is>
       </c>
     </row>
@@ -4092,96 +4082,76 @@
       </c>
       <c r="B167" t="inlineStr">
         <is>
-          <t xml:space="preserve">Anbefalte</t>
+          <t xml:space="preserve">Referanse</t>
         </is>
       </c>
       <c r="C167" t="inlineStr">
         <is>
-          <t xml:space="preserve">recommended</t>
+          <t xml:space="preserve">reference</t>
         </is>
       </c>
       <c r="D167" t="inlineStr">
         <is>
-          <t xml:space="preserve">list</t>
+          <t xml:space="preserve">text</t>
         </is>
       </c>
       <c r="G167" t="inlineStr">
         <is>
-          <t xml:space="preserve">IFC4</t>
+          <t xml:space="preserve">BEP §3</t>
         </is>
       </c>
     </row>
     <row r="168">
       <c r="A168" t="inlineStr">
         <is>
-          <t xml:space="preserve">Kilder</t>
+          <t xml:space="preserve">Standardkrav</t>
         </is>
       </c>
       <c r="B168" t="inlineStr">
         <is>
-          <t xml:space="preserve">Krav</t>
+          <t xml:space="preserve">Godtatte</t>
         </is>
       </c>
       <c r="C168" t="inlineStr">
         <is>
-          <t xml:space="preserve">projectLayer</t>
+          <t xml:space="preserve">accepted</t>
         </is>
       </c>
       <c r="D168" t="inlineStr">
         <is>
-          <t xml:space="preserve">text</t>
-        </is>
-      </c>
-      <c r="E168" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
-        </is>
-      </c>
-      <c r="F168" t="inlineStr">
-        <is>
-          <t xml:space="preserve">phase.sources, material-product.mengdetype, material-product.product, material-product.material</t>
+          <t xml:space="preserve">list</t>
         </is>
       </c>
       <c r="G168" t="inlineStr">
         <is>
-          <t xml:space="preserve">phase.sources</t>
+          <t xml:space="preserve">IFC2X3, IFC4</t>
         </is>
       </c>
     </row>
     <row r="169">
       <c r="A169" t="inlineStr">
         <is>
-          <t xml:space="preserve">Kilder</t>
+          <t xml:space="preserve">Standardkrav</t>
         </is>
       </c>
       <c r="B169" t="inlineStr">
         <is>
-          <t xml:space="preserve">Kildetype</t>
+          <t xml:space="preserve">Anbefalte</t>
         </is>
       </c>
       <c r="C169" t="inlineStr">
         <is>
-          <t xml:space="preserve">source</t>
+          <t xml:space="preserve">recommended</t>
         </is>
       </c>
       <c r="D169" t="inlineStr">
         <is>
-          <t xml:space="preserve">source kind</t>
-        </is>
-      </c>
-      <c r="E169" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
-        </is>
-      </c>
-      <c r="F169" t="inlineStr">
-        <is>
-          <t xml:space="preserve">attribute, property, classification, material, progressCode</t>
+          <t xml:space="preserve">list</t>
         </is>
       </c>
       <c r="G169" t="inlineStr">
         <is>
-          <t xml:space="preserve">property</t>
+          <t xml:space="preserve">IFC4</t>
         </is>
       </c>
     </row>
@@ -4193,12 +4163,12 @@
       </c>
       <c r="B170" t="inlineStr">
         <is>
-          <t xml:space="preserve">Attributt</t>
+          <t xml:space="preserve">Krav</t>
         </is>
       </c>
       <c r="C170" t="inlineStr">
         <is>
-          <t xml:space="preserve">source.attribute</t>
+          <t xml:space="preserve">projectLayer</t>
         </is>
       </c>
       <c r="D170" t="inlineStr">
@@ -4206,9 +4176,19 @@
           <t xml:space="preserve">text</t>
         </is>
       </c>
+      <c r="E170" t="inlineStr">
+        <is>
+          <t xml:space="preserve">yes</t>
+        </is>
+      </c>
+      <c r="F170" t="inlineStr">
+        <is>
+          <t xml:space="preserve">phase.sources, material-product.mengdetype, material-product.product, material-product.material</t>
+        </is>
+      </c>
       <c r="G170" t="inlineStr">
         <is>
-          <t xml:space="preserve">Name</t>
+          <t xml:space="preserve">phase.sources</t>
         </is>
       </c>
     </row>
@@ -4220,22 +4200,32 @@
       </c>
       <c r="B171" t="inlineStr">
         <is>
-          <t xml:space="preserve">Egenskapssett</t>
+          <t xml:space="preserve">Kildetype</t>
         </is>
       </c>
       <c r="C171" t="inlineStr">
         <is>
-          <t xml:space="preserve">source.property.propertySet</t>
+          <t xml:space="preserve">source</t>
         </is>
       </c>
       <c r="D171" t="inlineStr">
         <is>
-          <t xml:space="preserve">text</t>
+          <t xml:space="preserve">source kind</t>
+        </is>
+      </c>
+      <c r="E171" t="inlineStr">
+        <is>
+          <t xml:space="preserve">yes</t>
+        </is>
+      </c>
+      <c r="F171" t="inlineStr">
+        <is>
+          <t xml:space="preserve">attribute, property, classification, material, progressCode</t>
         </is>
       </c>
       <c r="G171" t="inlineStr">
         <is>
-          <t xml:space="preserve">EKS_Project</t>
+          <t xml:space="preserve">property</t>
         </is>
       </c>
     </row>
@@ -4247,12 +4237,12 @@
       </c>
       <c r="B172" t="inlineStr">
         <is>
-          <t xml:space="preserve">Egenskapsnavn</t>
+          <t xml:space="preserve">Attributt</t>
         </is>
       </c>
       <c r="C172" t="inlineStr">
         <is>
-          <t xml:space="preserve">source.property.name</t>
+          <t xml:space="preserve">source.attribute</t>
         </is>
       </c>
       <c r="D172" t="inlineStr">
@@ -4262,7 +4252,7 @@
       </c>
       <c r="G172" t="inlineStr">
         <is>
-          <t xml:space="preserve">MMI</t>
+          <t xml:space="preserve">Name</t>
         </is>
       </c>
     </row>
@@ -4274,12 +4264,12 @@
       </c>
       <c r="B173" t="inlineStr">
         <is>
-          <t xml:space="preserve">System</t>
+          <t xml:space="preserve">Egenskapssett</t>
         </is>
       </c>
       <c r="C173" t="inlineStr">
         <is>
-          <t xml:space="preserve">source.classification.system</t>
+          <t xml:space="preserve">source.property.propertySet</t>
         </is>
       </c>
       <c r="D173" t="inlineStr">
@@ -4289,37 +4279,91 @@
       </c>
       <c r="G173" t="inlineStr">
         <is>
-          <t xml:space="preserve">NS 3451</t>
+          <t xml:space="preserve">EKS_Project</t>
         </is>
       </c>
     </row>
     <row r="174">
       <c r="A174" t="inlineStr">
         <is>
+          <t xml:space="preserve">Kilder</t>
+        </is>
+      </c>
+      <c r="B174" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Egenskapsnavn</t>
+        </is>
+      </c>
+      <c r="C174" t="inlineStr">
+        <is>
+          <t xml:space="preserve">source.property.name</t>
+        </is>
+      </c>
+      <c r="D174" t="inlineStr">
+        <is>
+          <t xml:space="preserve">text</t>
+        </is>
+      </c>
+      <c r="G174" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MMI</t>
+        </is>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Kilder</t>
+        </is>
+      </c>
+      <c r="B175" t="inlineStr">
+        <is>
+          <t xml:space="preserve">System</t>
+        </is>
+      </c>
+      <c r="C175" t="inlineStr">
+        <is>
+          <t xml:space="preserve">source.classification.system</t>
+        </is>
+      </c>
+      <c r="D175" t="inlineStr">
+        <is>
+          <t xml:space="preserve">text</t>
+        </is>
+      </c>
+      <c r="G175" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NS 3451</t>
+        </is>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" t="inlineStr">
+        <is>
           <t xml:space="preserve">Andre regler</t>
         </is>
       </c>
-      <c r="B174" t="inlineStr">
+      <c r="B176" t="inlineStr">
         <is>
           <t xml:space="preserve">Regel</t>
         </is>
       </c>
-      <c r="C174" t="inlineStr">
+      <c r="C176" t="inlineStr">
         <is>
           <t xml:space="preserve">rules[]</t>
         </is>
       </c>
-      <c r="D174" t="inlineStr">
+      <c r="D176" t="inlineStr">
         <is>
           <t xml:space="preserve">JSON</t>
         </is>
       </c>
-      <c r="E174" t="inlineStr">
+      <c r="E176" t="inlineStr">
         <is>
           <t xml:space="preserve">yes</t>
         </is>
       </c>
-      <c r="G174" t="inlineStr">
+      <c r="G176" t="inlineStr">
         <is>
           <t xml:space="preserve">{"id":"elements-typed","kind":"extended","name":"Typed","select":{"entity":{"group":"physicalElement"}},"check":{"type":"element-typed"}}</t>
         </is>
@@ -4802,15 +4846,16 @@
     <col min="2" max="2" width="16" customWidth="1"/>
     <col min="3" max="3" width="16" customWidth="1"/>
     <col min="4" max="4" width="15" customWidth="1"/>
-    <col min="5" max="5" width="12" customWidth="1"/>
-    <col min="6" max="6" width="14" customWidth="1"/>
-    <col min="7" max="7" width="18" customWidth="1"/>
-    <col min="8" max="8" width="13" customWidth="1"/>
-    <col min="9" max="9" width="11" customWidth="1"/>
-    <col min="10" max="10" width="14" customWidth="1"/>
-    <col min="11" max="11" width="16" customWidth="1"/>
+    <col min="5" max="5" width="16" customWidth="1"/>
+    <col min="6" max="6" width="12" customWidth="1"/>
+    <col min="7" max="7" width="14" customWidth="1"/>
+    <col min="8" max="8" width="18" customWidth="1"/>
+    <col min="9" max="9" width="13" customWidth="1"/>
+    <col min="10" max="10" width="11" customWidth="1"/>
+    <col min="11" max="11" width="14" customWidth="1"/>
     <col min="12" max="12" width="16" customWidth="1"/>
-    <col min="13" max="13" width="13" customWidth="1"/>
+    <col min="13" max="13" width="16" customWidth="1"/>
+    <col min="14" max="14" width="13" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -4836,45 +4881,50 @@
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
+          <t xml:space="preserve">Ignorert</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
           <t xml:space="preserve">Tittel</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">Versjon</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">IDS-beskrivelse</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">Forfatter</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">Dato</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">Formål</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">Milepæl</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">Opphavsrett</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">JSON-skjema</t>
         </is>
@@ -4903,45 +4953,50 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
+          <t xml:space="preserve">ignore</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
           <t xml:space="preserve">info.title</t>
         </is>
       </c>
-      <c r="F2" s="2" t="inlineStr">
+      <c r="G2" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">info.version</t>
         </is>
       </c>
-      <c r="G2" s="2" t="inlineStr">
+      <c r="H2" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">info.description</t>
         </is>
       </c>
-      <c r="H2" s="2" t="inlineStr">
+      <c r="I2" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">info.author</t>
         </is>
       </c>
-      <c r="I2" s="2" t="inlineStr">
+      <c r="J2" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">info.date</t>
         </is>
       </c>
-      <c r="J2" s="2" t="inlineStr">
+      <c r="K2" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">info.purpose</t>
         </is>
       </c>
-      <c r="K2" s="2" t="inlineStr">
+      <c r="L2" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">info.milestone</t>
         </is>
       </c>
-      <c r="L2" s="2" t="inlineStr">
+      <c r="M2" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">info.copyright</t>
         </is>
       </c>
-      <c r="M2" s="2" t="inlineStr">
+      <c r="N2" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">$schema</t>
         </is>
@@ -4964,6 +5019,11 @@
       <c r="D3" t="inlineStr">
         <is>
           <t xml:space="preserve">IFC2X3, IFC4</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&lt;FROM PROJECT&gt;</t>
         </is>
       </c>
     </row>

</xml_diff>